<commit_message>
feat(generator): add validated sample change records
</commit_message>
<xml_diff>
--- a/docs/engineering/change-management/PO-CHANGE-REGISTER_v1.0.xlsx
+++ b/docs/engineering/change-management/PO-CHANGE-REGISTER_v1.0.xlsx
@@ -91,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -105,6 +105,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -668,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S4"/>
+  <dimension ref="A1:S503"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -804,25 +805,3245 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
-      <c r="M4" s="6" t="n"/>
-      <c r="N4" s="6" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>CHG-000001</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Upgrade Core Firewall Firmware</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>CI-NET-001</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>AST-NET-001</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Infrastructure Team</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Network Engineer</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="n">
+        <v>46286.83333333334</v>
+      </c>
+      <c r="N4" s="6" t="n">
+        <v>46286.91666666666</v>
+      </c>
       <c r="O4" s="6" t="n"/>
       <c r="P4" s="6" t="n"/>
-      <c r="Q4" s="5" t="n"/>
-      <c r="R4" s="5" t="n"/>
-      <c r="S4" s="5" t="n"/>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>Scheduled maintenance window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CHG-000002</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Patch Windows Domain Controller</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Server</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>CI-SRV-001</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>AST-SRV-001</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Security Team</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Systems Engineer</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>46287.79166666666</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>46287.875</v>
+      </c>
+      <c r="O5" s="7" t="n"/>
+      <c r="P5" s="7" t="n"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Security patch deployment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CHG-000003</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Rotate Cloud Service Credentials</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Cloud</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>CI-CLD-001</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>AST-CLD-001</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Cloud Operations</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Cloud Engineer</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>46280.75</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>46280.79166666666</v>
+      </c>
+      <c r="O6" s="7" t="n">
+        <v>46280.75347222222</v>
+      </c>
+      <c r="P6" s="7" t="n">
+        <v>46280.78333333333</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Change completed and validated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="M7" s="7" t="n"/>
+      <c r="N7" s="7" t="n"/>
+      <c r="O7" s="7" t="n"/>
+      <c r="P7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="M8" s="7" t="n"/>
+      <c r="N8" s="7" t="n"/>
+      <c r="O8" s="7" t="n"/>
+      <c r="P8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="M9" s="7" t="n"/>
+      <c r="N9" s="7" t="n"/>
+      <c r="O9" s="7" t="n"/>
+      <c r="P9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="M10" s="7" t="n"/>
+      <c r="N10" s="7" t="n"/>
+      <c r="O10" s="7" t="n"/>
+      <c r="P10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="M11" s="7" t="n"/>
+      <c r="N11" s="7" t="n"/>
+      <c r="O11" s="7" t="n"/>
+      <c r="P11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="M12" s="7" t="n"/>
+      <c r="N12" s="7" t="n"/>
+      <c r="O12" s="7" t="n"/>
+      <c r="P12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="M13" s="7" t="n"/>
+      <c r="N13" s="7" t="n"/>
+      <c r="O13" s="7" t="n"/>
+      <c r="P13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="M14" s="7" t="n"/>
+      <c r="N14" s="7" t="n"/>
+      <c r="O14" s="7" t="n"/>
+      <c r="P14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="M15" s="7" t="n"/>
+      <c r="N15" s="7" t="n"/>
+      <c r="O15" s="7" t="n"/>
+      <c r="P15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="M16" s="7" t="n"/>
+      <c r="N16" s="7" t="n"/>
+      <c r="O16" s="7" t="n"/>
+      <c r="P16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="M17" s="7" t="n"/>
+      <c r="N17" s="7" t="n"/>
+      <c r="O17" s="7" t="n"/>
+      <c r="P17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="M18" s="7" t="n"/>
+      <c r="N18" s="7" t="n"/>
+      <c r="O18" s="7" t="n"/>
+      <c r="P18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="M19" s="7" t="n"/>
+      <c r="N19" s="7" t="n"/>
+      <c r="O19" s="7" t="n"/>
+      <c r="P19" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="M20" s="7" t="n"/>
+      <c r="N20" s="7" t="n"/>
+      <c r="O20" s="7" t="n"/>
+      <c r="P20" s="7" t="n"/>
+    </row>
+    <row r="21">
+      <c r="M21" s="7" t="n"/>
+      <c r="N21" s="7" t="n"/>
+      <c r="O21" s="7" t="n"/>
+      <c r="P21" s="7" t="n"/>
+    </row>
+    <row r="22">
+      <c r="M22" s="7" t="n"/>
+      <c r="N22" s="7" t="n"/>
+      <c r="O22" s="7" t="n"/>
+      <c r="P22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="M23" s="7" t="n"/>
+      <c r="N23" s="7" t="n"/>
+      <c r="O23" s="7" t="n"/>
+      <c r="P23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="M24" s="7" t="n"/>
+      <c r="N24" s="7" t="n"/>
+      <c r="O24" s="7" t="n"/>
+      <c r="P24" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="M25" s="7" t="n"/>
+      <c r="N25" s="7" t="n"/>
+      <c r="O25" s="7" t="n"/>
+      <c r="P25" s="7" t="n"/>
+    </row>
+    <row r="26">
+      <c r="M26" s="7" t="n"/>
+      <c r="N26" s="7" t="n"/>
+      <c r="O26" s="7" t="n"/>
+      <c r="P26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="M27" s="7" t="n"/>
+      <c r="N27" s="7" t="n"/>
+      <c r="O27" s="7" t="n"/>
+      <c r="P27" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="M28" s="7" t="n"/>
+      <c r="N28" s="7" t="n"/>
+      <c r="O28" s="7" t="n"/>
+      <c r="P28" s="7" t="n"/>
+    </row>
+    <row r="29">
+      <c r="M29" s="7" t="n"/>
+      <c r="N29" s="7" t="n"/>
+      <c r="O29" s="7" t="n"/>
+      <c r="P29" s="7" t="n"/>
+    </row>
+    <row r="30">
+      <c r="M30" s="7" t="n"/>
+      <c r="N30" s="7" t="n"/>
+      <c r="O30" s="7" t="n"/>
+      <c r="P30" s="7" t="n"/>
+    </row>
+    <row r="31">
+      <c r="M31" s="7" t="n"/>
+      <c r="N31" s="7" t="n"/>
+      <c r="O31" s="7" t="n"/>
+      <c r="P31" s="7" t="n"/>
+    </row>
+    <row r="32">
+      <c r="M32" s="7" t="n"/>
+      <c r="N32" s="7" t="n"/>
+      <c r="O32" s="7" t="n"/>
+      <c r="P32" s="7" t="n"/>
+    </row>
+    <row r="33">
+      <c r="M33" s="7" t="n"/>
+      <c r="N33" s="7" t="n"/>
+      <c r="O33" s="7" t="n"/>
+      <c r="P33" s="7" t="n"/>
+    </row>
+    <row r="34">
+      <c r="M34" s="7" t="n"/>
+      <c r="N34" s="7" t="n"/>
+      <c r="O34" s="7" t="n"/>
+      <c r="P34" s="7" t="n"/>
+    </row>
+    <row r="35">
+      <c r="M35" s="7" t="n"/>
+      <c r="N35" s="7" t="n"/>
+      <c r="O35" s="7" t="n"/>
+      <c r="P35" s="7" t="n"/>
+    </row>
+    <row r="36">
+      <c r="M36" s="7" t="n"/>
+      <c r="N36" s="7" t="n"/>
+      <c r="O36" s="7" t="n"/>
+      <c r="P36" s="7" t="n"/>
+    </row>
+    <row r="37">
+      <c r="M37" s="7" t="n"/>
+      <c r="N37" s="7" t="n"/>
+      <c r="O37" s="7" t="n"/>
+      <c r="P37" s="7" t="n"/>
+    </row>
+    <row r="38">
+      <c r="M38" s="7" t="n"/>
+      <c r="N38" s="7" t="n"/>
+      <c r="O38" s="7" t="n"/>
+      <c r="P38" s="7" t="n"/>
+    </row>
+    <row r="39">
+      <c r="M39" s="7" t="n"/>
+      <c r="N39" s="7" t="n"/>
+      <c r="O39" s="7" t="n"/>
+      <c r="P39" s="7" t="n"/>
+    </row>
+    <row r="40">
+      <c r="M40" s="7" t="n"/>
+      <c r="N40" s="7" t="n"/>
+      <c r="O40" s="7" t="n"/>
+      <c r="P40" s="7" t="n"/>
+    </row>
+    <row r="41">
+      <c r="M41" s="7" t="n"/>
+      <c r="N41" s="7" t="n"/>
+      <c r="O41" s="7" t="n"/>
+      <c r="P41" s="7" t="n"/>
+    </row>
+    <row r="42">
+      <c r="M42" s="7" t="n"/>
+      <c r="N42" s="7" t="n"/>
+      <c r="O42" s="7" t="n"/>
+      <c r="P42" s="7" t="n"/>
+    </row>
+    <row r="43">
+      <c r="M43" s="7" t="n"/>
+      <c r="N43" s="7" t="n"/>
+      <c r="O43" s="7" t="n"/>
+      <c r="P43" s="7" t="n"/>
+    </row>
+    <row r="44">
+      <c r="M44" s="7" t="n"/>
+      <c r="N44" s="7" t="n"/>
+      <c r="O44" s="7" t="n"/>
+      <c r="P44" s="7" t="n"/>
+    </row>
+    <row r="45">
+      <c r="M45" s="7" t="n"/>
+      <c r="N45" s="7" t="n"/>
+      <c r="O45" s="7" t="n"/>
+      <c r="P45" s="7" t="n"/>
+    </row>
+    <row r="46">
+      <c r="M46" s="7" t="n"/>
+      <c r="N46" s="7" t="n"/>
+      <c r="O46" s="7" t="n"/>
+      <c r="P46" s="7" t="n"/>
+    </row>
+    <row r="47">
+      <c r="M47" s="7" t="n"/>
+      <c r="N47" s="7" t="n"/>
+      <c r="O47" s="7" t="n"/>
+      <c r="P47" s="7" t="n"/>
+    </row>
+    <row r="48">
+      <c r="M48" s="7" t="n"/>
+      <c r="N48" s="7" t="n"/>
+      <c r="O48" s="7" t="n"/>
+      <c r="P48" s="7" t="n"/>
+    </row>
+    <row r="49">
+      <c r="M49" s="7" t="n"/>
+      <c r="N49" s="7" t="n"/>
+      <c r="O49" s="7" t="n"/>
+      <c r="P49" s="7" t="n"/>
+    </row>
+    <row r="50">
+      <c r="M50" s="7" t="n"/>
+      <c r="N50" s="7" t="n"/>
+      <c r="O50" s="7" t="n"/>
+      <c r="P50" s="7" t="n"/>
+    </row>
+    <row r="51">
+      <c r="M51" s="7" t="n"/>
+      <c r="N51" s="7" t="n"/>
+      <c r="O51" s="7" t="n"/>
+      <c r="P51" s="7" t="n"/>
+    </row>
+    <row r="52">
+      <c r="M52" s="7" t="n"/>
+      <c r="N52" s="7" t="n"/>
+      <c r="O52" s="7" t="n"/>
+      <c r="P52" s="7" t="n"/>
+    </row>
+    <row r="53">
+      <c r="M53" s="7" t="n"/>
+      <c r="N53" s="7" t="n"/>
+      <c r="O53" s="7" t="n"/>
+      <c r="P53" s="7" t="n"/>
+    </row>
+    <row r="54">
+      <c r="M54" s="7" t="n"/>
+      <c r="N54" s="7" t="n"/>
+      <c r="O54" s="7" t="n"/>
+      <c r="P54" s="7" t="n"/>
+    </row>
+    <row r="55">
+      <c r="M55" s="7" t="n"/>
+      <c r="N55" s="7" t="n"/>
+      <c r="O55" s="7" t="n"/>
+      <c r="P55" s="7" t="n"/>
+    </row>
+    <row r="56">
+      <c r="M56" s="7" t="n"/>
+      <c r="N56" s="7" t="n"/>
+      <c r="O56" s="7" t="n"/>
+      <c r="P56" s="7" t="n"/>
+    </row>
+    <row r="57">
+      <c r="M57" s="7" t="n"/>
+      <c r="N57" s="7" t="n"/>
+      <c r="O57" s="7" t="n"/>
+      <c r="P57" s="7" t="n"/>
+    </row>
+    <row r="58">
+      <c r="M58" s="7" t="n"/>
+      <c r="N58" s="7" t="n"/>
+      <c r="O58" s="7" t="n"/>
+      <c r="P58" s="7" t="n"/>
+    </row>
+    <row r="59">
+      <c r="M59" s="7" t="n"/>
+      <c r="N59" s="7" t="n"/>
+      <c r="O59" s="7" t="n"/>
+      <c r="P59" s="7" t="n"/>
+    </row>
+    <row r="60">
+      <c r="M60" s="7" t="n"/>
+      <c r="N60" s="7" t="n"/>
+      <c r="O60" s="7" t="n"/>
+      <c r="P60" s="7" t="n"/>
+    </row>
+    <row r="61">
+      <c r="M61" s="7" t="n"/>
+      <c r="N61" s="7" t="n"/>
+      <c r="O61" s="7" t="n"/>
+      <c r="P61" s="7" t="n"/>
+    </row>
+    <row r="62">
+      <c r="M62" s="7" t="n"/>
+      <c r="N62" s="7" t="n"/>
+      <c r="O62" s="7" t="n"/>
+      <c r="P62" s="7" t="n"/>
+    </row>
+    <row r="63">
+      <c r="M63" s="7" t="n"/>
+      <c r="N63" s="7" t="n"/>
+      <c r="O63" s="7" t="n"/>
+      <c r="P63" s="7" t="n"/>
+    </row>
+    <row r="64">
+      <c r="M64" s="7" t="n"/>
+      <c r="N64" s="7" t="n"/>
+      <c r="O64" s="7" t="n"/>
+      <c r="P64" s="7" t="n"/>
+    </row>
+    <row r="65">
+      <c r="M65" s="7" t="n"/>
+      <c r="N65" s="7" t="n"/>
+      <c r="O65" s="7" t="n"/>
+      <c r="P65" s="7" t="n"/>
+    </row>
+    <row r="66">
+      <c r="M66" s="7" t="n"/>
+      <c r="N66" s="7" t="n"/>
+      <c r="O66" s="7" t="n"/>
+      <c r="P66" s="7" t="n"/>
+    </row>
+    <row r="67">
+      <c r="M67" s="7" t="n"/>
+      <c r="N67" s="7" t="n"/>
+      <c r="O67" s="7" t="n"/>
+      <c r="P67" s="7" t="n"/>
+    </row>
+    <row r="68">
+      <c r="M68" s="7" t="n"/>
+      <c r="N68" s="7" t="n"/>
+      <c r="O68" s="7" t="n"/>
+      <c r="P68" s="7" t="n"/>
+    </row>
+    <row r="69">
+      <c r="M69" s="7" t="n"/>
+      <c r="N69" s="7" t="n"/>
+      <c r="O69" s="7" t="n"/>
+      <c r="P69" s="7" t="n"/>
+    </row>
+    <row r="70">
+      <c r="M70" s="7" t="n"/>
+      <c r="N70" s="7" t="n"/>
+      <c r="O70" s="7" t="n"/>
+      <c r="P70" s="7" t="n"/>
+    </row>
+    <row r="71">
+      <c r="M71" s="7" t="n"/>
+      <c r="N71" s="7" t="n"/>
+      <c r="O71" s="7" t="n"/>
+      <c r="P71" s="7" t="n"/>
+    </row>
+    <row r="72">
+      <c r="M72" s="7" t="n"/>
+      <c r="N72" s="7" t="n"/>
+      <c r="O72" s="7" t="n"/>
+      <c r="P72" s="7" t="n"/>
+    </row>
+    <row r="73">
+      <c r="M73" s="7" t="n"/>
+      <c r="N73" s="7" t="n"/>
+      <c r="O73" s="7" t="n"/>
+      <c r="P73" s="7" t="n"/>
+    </row>
+    <row r="74">
+      <c r="M74" s="7" t="n"/>
+      <c r="N74" s="7" t="n"/>
+      <c r="O74" s="7" t="n"/>
+      <c r="P74" s="7" t="n"/>
+    </row>
+    <row r="75">
+      <c r="M75" s="7" t="n"/>
+      <c r="N75" s="7" t="n"/>
+      <c r="O75" s="7" t="n"/>
+      <c r="P75" s="7" t="n"/>
+    </row>
+    <row r="76">
+      <c r="M76" s="7" t="n"/>
+      <c r="N76" s="7" t="n"/>
+      <c r="O76" s="7" t="n"/>
+      <c r="P76" s="7" t="n"/>
+    </row>
+    <row r="77">
+      <c r="M77" s="7" t="n"/>
+      <c r="N77" s="7" t="n"/>
+      <c r="O77" s="7" t="n"/>
+      <c r="P77" s="7" t="n"/>
+    </row>
+    <row r="78">
+      <c r="M78" s="7" t="n"/>
+      <c r="N78" s="7" t="n"/>
+      <c r="O78" s="7" t="n"/>
+      <c r="P78" s="7" t="n"/>
+    </row>
+    <row r="79">
+      <c r="M79" s="7" t="n"/>
+      <c r="N79" s="7" t="n"/>
+      <c r="O79" s="7" t="n"/>
+      <c r="P79" s="7" t="n"/>
+    </row>
+    <row r="80">
+      <c r="M80" s="7" t="n"/>
+      <c r="N80" s="7" t="n"/>
+      <c r="O80" s="7" t="n"/>
+      <c r="P80" s="7" t="n"/>
+    </row>
+    <row r="81">
+      <c r="M81" s="7" t="n"/>
+      <c r="N81" s="7" t="n"/>
+      <c r="O81" s="7" t="n"/>
+      <c r="P81" s="7" t="n"/>
+    </row>
+    <row r="82">
+      <c r="M82" s="7" t="n"/>
+      <c r="N82" s="7" t="n"/>
+      <c r="O82" s="7" t="n"/>
+      <c r="P82" s="7" t="n"/>
+    </row>
+    <row r="83">
+      <c r="M83" s="7" t="n"/>
+      <c r="N83" s="7" t="n"/>
+      <c r="O83" s="7" t="n"/>
+      <c r="P83" s="7" t="n"/>
+    </row>
+    <row r="84">
+      <c r="M84" s="7" t="n"/>
+      <c r="N84" s="7" t="n"/>
+      <c r="O84" s="7" t="n"/>
+      <c r="P84" s="7" t="n"/>
+    </row>
+    <row r="85">
+      <c r="M85" s="7" t="n"/>
+      <c r="N85" s="7" t="n"/>
+      <c r="O85" s="7" t="n"/>
+      <c r="P85" s="7" t="n"/>
+    </row>
+    <row r="86">
+      <c r="M86" s="7" t="n"/>
+      <c r="N86" s="7" t="n"/>
+      <c r="O86" s="7" t="n"/>
+      <c r="P86" s="7" t="n"/>
+    </row>
+    <row r="87">
+      <c r="M87" s="7" t="n"/>
+      <c r="N87" s="7" t="n"/>
+      <c r="O87" s="7" t="n"/>
+      <c r="P87" s="7" t="n"/>
+    </row>
+    <row r="88">
+      <c r="M88" s="7" t="n"/>
+      <c r="N88" s="7" t="n"/>
+      <c r="O88" s="7" t="n"/>
+      <c r="P88" s="7" t="n"/>
+    </row>
+    <row r="89">
+      <c r="M89" s="7" t="n"/>
+      <c r="N89" s="7" t="n"/>
+      <c r="O89" s="7" t="n"/>
+      <c r="P89" s="7" t="n"/>
+    </row>
+    <row r="90">
+      <c r="M90" s="7" t="n"/>
+      <c r="N90" s="7" t="n"/>
+      <c r="O90" s="7" t="n"/>
+      <c r="P90" s="7" t="n"/>
+    </row>
+    <row r="91">
+      <c r="M91" s="7" t="n"/>
+      <c r="N91" s="7" t="n"/>
+      <c r="O91" s="7" t="n"/>
+      <c r="P91" s="7" t="n"/>
+    </row>
+    <row r="92">
+      <c r="M92" s="7" t="n"/>
+      <c r="N92" s="7" t="n"/>
+      <c r="O92" s="7" t="n"/>
+      <c r="P92" s="7" t="n"/>
+    </row>
+    <row r="93">
+      <c r="M93" s="7" t="n"/>
+      <c r="N93" s="7" t="n"/>
+      <c r="O93" s="7" t="n"/>
+      <c r="P93" s="7" t="n"/>
+    </row>
+    <row r="94">
+      <c r="M94" s="7" t="n"/>
+      <c r="N94" s="7" t="n"/>
+      <c r="O94" s="7" t="n"/>
+      <c r="P94" s="7" t="n"/>
+    </row>
+    <row r="95">
+      <c r="M95" s="7" t="n"/>
+      <c r="N95" s="7" t="n"/>
+      <c r="O95" s="7" t="n"/>
+      <c r="P95" s="7" t="n"/>
+    </row>
+    <row r="96">
+      <c r="M96" s="7" t="n"/>
+      <c r="N96" s="7" t="n"/>
+      <c r="O96" s="7" t="n"/>
+      <c r="P96" s="7" t="n"/>
+    </row>
+    <row r="97">
+      <c r="M97" s="7" t="n"/>
+      <c r="N97" s="7" t="n"/>
+      <c r="O97" s="7" t="n"/>
+      <c r="P97" s="7" t="n"/>
+    </row>
+    <row r="98">
+      <c r="M98" s="7" t="n"/>
+      <c r="N98" s="7" t="n"/>
+      <c r="O98" s="7" t="n"/>
+      <c r="P98" s="7" t="n"/>
+    </row>
+    <row r="99">
+      <c r="M99" s="7" t="n"/>
+      <c r="N99" s="7" t="n"/>
+      <c r="O99" s="7" t="n"/>
+      <c r="P99" s="7" t="n"/>
+    </row>
+    <row r="100">
+      <c r="M100" s="7" t="n"/>
+      <c r="N100" s="7" t="n"/>
+      <c r="O100" s="7" t="n"/>
+      <c r="P100" s="7" t="n"/>
+    </row>
+    <row r="101">
+      <c r="M101" s="7" t="n"/>
+      <c r="N101" s="7" t="n"/>
+      <c r="O101" s="7" t="n"/>
+      <c r="P101" s="7" t="n"/>
+    </row>
+    <row r="102">
+      <c r="M102" s="7" t="n"/>
+      <c r="N102" s="7" t="n"/>
+      <c r="O102" s="7" t="n"/>
+      <c r="P102" s="7" t="n"/>
+    </row>
+    <row r="103">
+      <c r="M103" s="7" t="n"/>
+      <c r="N103" s="7" t="n"/>
+      <c r="O103" s="7" t="n"/>
+      <c r="P103" s="7" t="n"/>
+    </row>
+    <row r="104">
+      <c r="M104" s="7" t="n"/>
+      <c r="N104" s="7" t="n"/>
+      <c r="O104" s="7" t="n"/>
+      <c r="P104" s="7" t="n"/>
+    </row>
+    <row r="105">
+      <c r="M105" s="7" t="n"/>
+      <c r="N105" s="7" t="n"/>
+      <c r="O105" s="7" t="n"/>
+      <c r="P105" s="7" t="n"/>
+    </row>
+    <row r="106">
+      <c r="M106" s="7" t="n"/>
+      <c r="N106" s="7" t="n"/>
+      <c r="O106" s="7" t="n"/>
+      <c r="P106" s="7" t="n"/>
+    </row>
+    <row r="107">
+      <c r="M107" s="7" t="n"/>
+      <c r="N107" s="7" t="n"/>
+      <c r="O107" s="7" t="n"/>
+      <c r="P107" s="7" t="n"/>
+    </row>
+    <row r="108">
+      <c r="M108" s="7" t="n"/>
+      <c r="N108" s="7" t="n"/>
+      <c r="O108" s="7" t="n"/>
+      <c r="P108" s="7" t="n"/>
+    </row>
+    <row r="109">
+      <c r="M109" s="7" t="n"/>
+      <c r="N109" s="7" t="n"/>
+      <c r="O109" s="7" t="n"/>
+      <c r="P109" s="7" t="n"/>
+    </row>
+    <row r="110">
+      <c r="M110" s="7" t="n"/>
+      <c r="N110" s="7" t="n"/>
+      <c r="O110" s="7" t="n"/>
+      <c r="P110" s="7" t="n"/>
+    </row>
+    <row r="111">
+      <c r="M111" s="7" t="n"/>
+      <c r="N111" s="7" t="n"/>
+      <c r="O111" s="7" t="n"/>
+      <c r="P111" s="7" t="n"/>
+    </row>
+    <row r="112">
+      <c r="M112" s="7" t="n"/>
+      <c r="N112" s="7" t="n"/>
+      <c r="O112" s="7" t="n"/>
+      <c r="P112" s="7" t="n"/>
+    </row>
+    <row r="113">
+      <c r="M113" s="7" t="n"/>
+      <c r="N113" s="7" t="n"/>
+      <c r="O113" s="7" t="n"/>
+      <c r="P113" s="7" t="n"/>
+    </row>
+    <row r="114">
+      <c r="M114" s="7" t="n"/>
+      <c r="N114" s="7" t="n"/>
+      <c r="O114" s="7" t="n"/>
+      <c r="P114" s="7" t="n"/>
+    </row>
+    <row r="115">
+      <c r="M115" s="7" t="n"/>
+      <c r="N115" s="7" t="n"/>
+      <c r="O115" s="7" t="n"/>
+      <c r="P115" s="7" t="n"/>
+    </row>
+    <row r="116">
+      <c r="M116" s="7" t="n"/>
+      <c r="N116" s="7" t="n"/>
+      <c r="O116" s="7" t="n"/>
+      <c r="P116" s="7" t="n"/>
+    </row>
+    <row r="117">
+      <c r="M117" s="7" t="n"/>
+      <c r="N117" s="7" t="n"/>
+      <c r="O117" s="7" t="n"/>
+      <c r="P117" s="7" t="n"/>
+    </row>
+    <row r="118">
+      <c r="M118" s="7" t="n"/>
+      <c r="N118" s="7" t="n"/>
+      <c r="O118" s="7" t="n"/>
+      <c r="P118" s="7" t="n"/>
+    </row>
+    <row r="119">
+      <c r="M119" s="7" t="n"/>
+      <c r="N119" s="7" t="n"/>
+      <c r="O119" s="7" t="n"/>
+      <c r="P119" s="7" t="n"/>
+    </row>
+    <row r="120">
+      <c r="M120" s="7" t="n"/>
+      <c r="N120" s="7" t="n"/>
+      <c r="O120" s="7" t="n"/>
+      <c r="P120" s="7" t="n"/>
+    </row>
+    <row r="121">
+      <c r="M121" s="7" t="n"/>
+      <c r="N121" s="7" t="n"/>
+      <c r="O121" s="7" t="n"/>
+      <c r="P121" s="7" t="n"/>
+    </row>
+    <row r="122">
+      <c r="M122" s="7" t="n"/>
+      <c r="N122" s="7" t="n"/>
+      <c r="O122" s="7" t="n"/>
+      <c r="P122" s="7" t="n"/>
+    </row>
+    <row r="123">
+      <c r="M123" s="7" t="n"/>
+      <c r="N123" s="7" t="n"/>
+      <c r="O123" s="7" t="n"/>
+      <c r="P123" s="7" t="n"/>
+    </row>
+    <row r="124">
+      <c r="M124" s="7" t="n"/>
+      <c r="N124" s="7" t="n"/>
+      <c r="O124" s="7" t="n"/>
+      <c r="P124" s="7" t="n"/>
+    </row>
+    <row r="125">
+      <c r="M125" s="7" t="n"/>
+      <c r="N125" s="7" t="n"/>
+      <c r="O125" s="7" t="n"/>
+      <c r="P125" s="7" t="n"/>
+    </row>
+    <row r="126">
+      <c r="M126" s="7" t="n"/>
+      <c r="N126" s="7" t="n"/>
+      <c r="O126" s="7" t="n"/>
+      <c r="P126" s="7" t="n"/>
+    </row>
+    <row r="127">
+      <c r="M127" s="7" t="n"/>
+      <c r="N127" s="7" t="n"/>
+      <c r="O127" s="7" t="n"/>
+      <c r="P127" s="7" t="n"/>
+    </row>
+    <row r="128">
+      <c r="M128" s="7" t="n"/>
+      <c r="N128" s="7" t="n"/>
+      <c r="O128" s="7" t="n"/>
+      <c r="P128" s="7" t="n"/>
+    </row>
+    <row r="129">
+      <c r="M129" s="7" t="n"/>
+      <c r="N129" s="7" t="n"/>
+      <c r="O129" s="7" t="n"/>
+      <c r="P129" s="7" t="n"/>
+    </row>
+    <row r="130">
+      <c r="M130" s="7" t="n"/>
+      <c r="N130" s="7" t="n"/>
+      <c r="O130" s="7" t="n"/>
+      <c r="P130" s="7" t="n"/>
+    </row>
+    <row r="131">
+      <c r="M131" s="7" t="n"/>
+      <c r="N131" s="7" t="n"/>
+      <c r="O131" s="7" t="n"/>
+      <c r="P131" s="7" t="n"/>
+    </row>
+    <row r="132">
+      <c r="M132" s="7" t="n"/>
+      <c r="N132" s="7" t="n"/>
+      <c r="O132" s="7" t="n"/>
+      <c r="P132" s="7" t="n"/>
+    </row>
+    <row r="133">
+      <c r="M133" s="7" t="n"/>
+      <c r="N133" s="7" t="n"/>
+      <c r="O133" s="7" t="n"/>
+      <c r="P133" s="7" t="n"/>
+    </row>
+    <row r="134">
+      <c r="M134" s="7" t="n"/>
+      <c r="N134" s="7" t="n"/>
+      <c r="O134" s="7" t="n"/>
+      <c r="P134" s="7" t="n"/>
+    </row>
+    <row r="135">
+      <c r="M135" s="7" t="n"/>
+      <c r="N135" s="7" t="n"/>
+      <c r="O135" s="7" t="n"/>
+      <c r="P135" s="7" t="n"/>
+    </row>
+    <row r="136">
+      <c r="M136" s="7" t="n"/>
+      <c r="N136" s="7" t="n"/>
+      <c r="O136" s="7" t="n"/>
+      <c r="P136" s="7" t="n"/>
+    </row>
+    <row r="137">
+      <c r="M137" s="7" t="n"/>
+      <c r="N137" s="7" t="n"/>
+      <c r="O137" s="7" t="n"/>
+      <c r="P137" s="7" t="n"/>
+    </row>
+    <row r="138">
+      <c r="M138" s="7" t="n"/>
+      <c r="N138" s="7" t="n"/>
+      <c r="O138" s="7" t="n"/>
+      <c r="P138" s="7" t="n"/>
+    </row>
+    <row r="139">
+      <c r="M139" s="7" t="n"/>
+      <c r="N139" s="7" t="n"/>
+      <c r="O139" s="7" t="n"/>
+      <c r="P139" s="7" t="n"/>
+    </row>
+    <row r="140">
+      <c r="M140" s="7" t="n"/>
+      <c r="N140" s="7" t="n"/>
+      <c r="O140" s="7" t="n"/>
+      <c r="P140" s="7" t="n"/>
+    </row>
+    <row r="141">
+      <c r="M141" s="7" t="n"/>
+      <c r="N141" s="7" t="n"/>
+      <c r="O141" s="7" t="n"/>
+      <c r="P141" s="7" t="n"/>
+    </row>
+    <row r="142">
+      <c r="M142" s="7" t="n"/>
+      <c r="N142" s="7" t="n"/>
+      <c r="O142" s="7" t="n"/>
+      <c r="P142" s="7" t="n"/>
+    </row>
+    <row r="143">
+      <c r="M143" s="7" t="n"/>
+      <c r="N143" s="7" t="n"/>
+      <c r="O143" s="7" t="n"/>
+      <c r="P143" s="7" t="n"/>
+    </row>
+    <row r="144">
+      <c r="M144" s="7" t="n"/>
+      <c r="N144" s="7" t="n"/>
+      <c r="O144" s="7" t="n"/>
+      <c r="P144" s="7" t="n"/>
+    </row>
+    <row r="145">
+      <c r="M145" s="7" t="n"/>
+      <c r="N145" s="7" t="n"/>
+      <c r="O145" s="7" t="n"/>
+      <c r="P145" s="7" t="n"/>
+    </row>
+    <row r="146">
+      <c r="M146" s="7" t="n"/>
+      <c r="N146" s="7" t="n"/>
+      <c r="O146" s="7" t="n"/>
+      <c r="P146" s="7" t="n"/>
+    </row>
+    <row r="147">
+      <c r="M147" s="7" t="n"/>
+      <c r="N147" s="7" t="n"/>
+      <c r="O147" s="7" t="n"/>
+      <c r="P147" s="7" t="n"/>
+    </row>
+    <row r="148">
+      <c r="M148" s="7" t="n"/>
+      <c r="N148" s="7" t="n"/>
+      <c r="O148" s="7" t="n"/>
+      <c r="P148" s="7" t="n"/>
+    </row>
+    <row r="149">
+      <c r="M149" s="7" t="n"/>
+      <c r="N149" s="7" t="n"/>
+      <c r="O149" s="7" t="n"/>
+      <c r="P149" s="7" t="n"/>
+    </row>
+    <row r="150">
+      <c r="M150" s="7" t="n"/>
+      <c r="N150" s="7" t="n"/>
+      <c r="O150" s="7" t="n"/>
+      <c r="P150" s="7" t="n"/>
+    </row>
+    <row r="151">
+      <c r="M151" s="7" t="n"/>
+      <c r="N151" s="7" t="n"/>
+      <c r="O151" s="7" t="n"/>
+      <c r="P151" s="7" t="n"/>
+    </row>
+    <row r="152">
+      <c r="M152" s="7" t="n"/>
+      <c r="N152" s="7" t="n"/>
+      <c r="O152" s="7" t="n"/>
+      <c r="P152" s="7" t="n"/>
+    </row>
+    <row r="153">
+      <c r="M153" s="7" t="n"/>
+      <c r="N153" s="7" t="n"/>
+      <c r="O153" s="7" t="n"/>
+      <c r="P153" s="7" t="n"/>
+    </row>
+    <row r="154">
+      <c r="M154" s="7" t="n"/>
+      <c r="N154" s="7" t="n"/>
+      <c r="O154" s="7" t="n"/>
+      <c r="P154" s="7" t="n"/>
+    </row>
+    <row r="155">
+      <c r="M155" s="7" t="n"/>
+      <c r="N155" s="7" t="n"/>
+      <c r="O155" s="7" t="n"/>
+      <c r="P155" s="7" t="n"/>
+    </row>
+    <row r="156">
+      <c r="M156" s="7" t="n"/>
+      <c r="N156" s="7" t="n"/>
+      <c r="O156" s="7" t="n"/>
+      <c r="P156" s="7" t="n"/>
+    </row>
+    <row r="157">
+      <c r="M157" s="7" t="n"/>
+      <c r="N157" s="7" t="n"/>
+      <c r="O157" s="7" t="n"/>
+      <c r="P157" s="7" t="n"/>
+    </row>
+    <row r="158">
+      <c r="M158" s="7" t="n"/>
+      <c r="N158" s="7" t="n"/>
+      <c r="O158" s="7" t="n"/>
+      <c r="P158" s="7" t="n"/>
+    </row>
+    <row r="159">
+      <c r="M159" s="7" t="n"/>
+      <c r="N159" s="7" t="n"/>
+      <c r="O159" s="7" t="n"/>
+      <c r="P159" s="7" t="n"/>
+    </row>
+    <row r="160">
+      <c r="M160" s="7" t="n"/>
+      <c r="N160" s="7" t="n"/>
+      <c r="O160" s="7" t="n"/>
+      <c r="P160" s="7" t="n"/>
+    </row>
+    <row r="161">
+      <c r="M161" s="7" t="n"/>
+      <c r="N161" s="7" t="n"/>
+      <c r="O161" s="7" t="n"/>
+      <c r="P161" s="7" t="n"/>
+    </row>
+    <row r="162">
+      <c r="M162" s="7" t="n"/>
+      <c r="N162" s="7" t="n"/>
+      <c r="O162" s="7" t="n"/>
+      <c r="P162" s="7" t="n"/>
+    </row>
+    <row r="163">
+      <c r="M163" s="7" t="n"/>
+      <c r="N163" s="7" t="n"/>
+      <c r="O163" s="7" t="n"/>
+      <c r="P163" s="7" t="n"/>
+    </row>
+    <row r="164">
+      <c r="M164" s="7" t="n"/>
+      <c r="N164" s="7" t="n"/>
+      <c r="O164" s="7" t="n"/>
+      <c r="P164" s="7" t="n"/>
+    </row>
+    <row r="165">
+      <c r="M165" s="7" t="n"/>
+      <c r="N165" s="7" t="n"/>
+      <c r="O165" s="7" t="n"/>
+      <c r="P165" s="7" t="n"/>
+    </row>
+    <row r="166">
+      <c r="M166" s="7" t="n"/>
+      <c r="N166" s="7" t="n"/>
+      <c r="O166" s="7" t="n"/>
+      <c r="P166" s="7" t="n"/>
+    </row>
+    <row r="167">
+      <c r="M167" s="7" t="n"/>
+      <c r="N167" s="7" t="n"/>
+      <c r="O167" s="7" t="n"/>
+      <c r="P167" s="7" t="n"/>
+    </row>
+    <row r="168">
+      <c r="M168" s="7" t="n"/>
+      <c r="N168" s="7" t="n"/>
+      <c r="O168" s="7" t="n"/>
+      <c r="P168" s="7" t="n"/>
+    </row>
+    <row r="169">
+      <c r="M169" s="7" t="n"/>
+      <c r="N169" s="7" t="n"/>
+      <c r="O169" s="7" t="n"/>
+      <c r="P169" s="7" t="n"/>
+    </row>
+    <row r="170">
+      <c r="M170" s="7" t="n"/>
+      <c r="N170" s="7" t="n"/>
+      <c r="O170" s="7" t="n"/>
+      <c r="P170" s="7" t="n"/>
+    </row>
+    <row r="171">
+      <c r="M171" s="7" t="n"/>
+      <c r="N171" s="7" t="n"/>
+      <c r="O171" s="7" t="n"/>
+      <c r="P171" s="7" t="n"/>
+    </row>
+    <row r="172">
+      <c r="M172" s="7" t="n"/>
+      <c r="N172" s="7" t="n"/>
+      <c r="O172" s="7" t="n"/>
+      <c r="P172" s="7" t="n"/>
+    </row>
+    <row r="173">
+      <c r="M173" s="7" t="n"/>
+      <c r="N173" s="7" t="n"/>
+      <c r="O173" s="7" t="n"/>
+      <c r="P173" s="7" t="n"/>
+    </row>
+    <row r="174">
+      <c r="M174" s="7" t="n"/>
+      <c r="N174" s="7" t="n"/>
+      <c r="O174" s="7" t="n"/>
+      <c r="P174" s="7" t="n"/>
+    </row>
+    <row r="175">
+      <c r="M175" s="7" t="n"/>
+      <c r="N175" s="7" t="n"/>
+      <c r="O175" s="7" t="n"/>
+      <c r="P175" s="7" t="n"/>
+    </row>
+    <row r="176">
+      <c r="M176" s="7" t="n"/>
+      <c r="N176" s="7" t="n"/>
+      <c r="O176" s="7" t="n"/>
+      <c r="P176" s="7" t="n"/>
+    </row>
+    <row r="177">
+      <c r="M177" s="7" t="n"/>
+      <c r="N177" s="7" t="n"/>
+      <c r="O177" s="7" t="n"/>
+      <c r="P177" s="7" t="n"/>
+    </row>
+    <row r="178">
+      <c r="M178" s="7" t="n"/>
+      <c r="N178" s="7" t="n"/>
+      <c r="O178" s="7" t="n"/>
+      <c r="P178" s="7" t="n"/>
+    </row>
+    <row r="179">
+      <c r="M179" s="7" t="n"/>
+      <c r="N179" s="7" t="n"/>
+      <c r="O179" s="7" t="n"/>
+      <c r="P179" s="7" t="n"/>
+    </row>
+    <row r="180">
+      <c r="M180" s="7" t="n"/>
+      <c r="N180" s="7" t="n"/>
+      <c r="O180" s="7" t="n"/>
+      <c r="P180" s="7" t="n"/>
+    </row>
+    <row r="181">
+      <c r="M181" s="7" t="n"/>
+      <c r="N181" s="7" t="n"/>
+      <c r="O181" s="7" t="n"/>
+      <c r="P181" s="7" t="n"/>
+    </row>
+    <row r="182">
+      <c r="M182" s="7" t="n"/>
+      <c r="N182" s="7" t="n"/>
+      <c r="O182" s="7" t="n"/>
+      <c r="P182" s="7" t="n"/>
+    </row>
+    <row r="183">
+      <c r="M183" s="7" t="n"/>
+      <c r="N183" s="7" t="n"/>
+      <c r="O183" s="7" t="n"/>
+      <c r="P183" s="7" t="n"/>
+    </row>
+    <row r="184">
+      <c r="M184" s="7" t="n"/>
+      <c r="N184" s="7" t="n"/>
+      <c r="O184" s="7" t="n"/>
+      <c r="P184" s="7" t="n"/>
+    </row>
+    <row r="185">
+      <c r="M185" s="7" t="n"/>
+      <c r="N185" s="7" t="n"/>
+      <c r="O185" s="7" t="n"/>
+      <c r="P185" s="7" t="n"/>
+    </row>
+    <row r="186">
+      <c r="M186" s="7" t="n"/>
+      <c r="N186" s="7" t="n"/>
+      <c r="O186" s="7" t="n"/>
+      <c r="P186" s="7" t="n"/>
+    </row>
+    <row r="187">
+      <c r="M187" s="7" t="n"/>
+      <c r="N187" s="7" t="n"/>
+      <c r="O187" s="7" t="n"/>
+      <c r="P187" s="7" t="n"/>
+    </row>
+    <row r="188">
+      <c r="M188" s="7" t="n"/>
+      <c r="N188" s="7" t="n"/>
+      <c r="O188" s="7" t="n"/>
+      <c r="P188" s="7" t="n"/>
+    </row>
+    <row r="189">
+      <c r="M189" s="7" t="n"/>
+      <c r="N189" s="7" t="n"/>
+      <c r="O189" s="7" t="n"/>
+      <c r="P189" s="7" t="n"/>
+    </row>
+    <row r="190">
+      <c r="M190" s="7" t="n"/>
+      <c r="N190" s="7" t="n"/>
+      <c r="O190" s="7" t="n"/>
+      <c r="P190" s="7" t="n"/>
+    </row>
+    <row r="191">
+      <c r="M191" s="7" t="n"/>
+      <c r="N191" s="7" t="n"/>
+      <c r="O191" s="7" t="n"/>
+      <c r="P191" s="7" t="n"/>
+    </row>
+    <row r="192">
+      <c r="M192" s="7" t="n"/>
+      <c r="N192" s="7" t="n"/>
+      <c r="O192" s="7" t="n"/>
+      <c r="P192" s="7" t="n"/>
+    </row>
+    <row r="193">
+      <c r="M193" s="7" t="n"/>
+      <c r="N193" s="7" t="n"/>
+      <c r="O193" s="7" t="n"/>
+      <c r="P193" s="7" t="n"/>
+    </row>
+    <row r="194">
+      <c r="M194" s="7" t="n"/>
+      <c r="N194" s="7" t="n"/>
+      <c r="O194" s="7" t="n"/>
+      <c r="P194" s="7" t="n"/>
+    </row>
+    <row r="195">
+      <c r="M195" s="7" t="n"/>
+      <c r="N195" s="7" t="n"/>
+      <c r="O195" s="7" t="n"/>
+      <c r="P195" s="7" t="n"/>
+    </row>
+    <row r="196">
+      <c r="M196" s="7" t="n"/>
+      <c r="N196" s="7" t="n"/>
+      <c r="O196" s="7" t="n"/>
+      <c r="P196" s="7" t="n"/>
+    </row>
+    <row r="197">
+      <c r="M197" s="7" t="n"/>
+      <c r="N197" s="7" t="n"/>
+      <c r="O197" s="7" t="n"/>
+      <c r="P197" s="7" t="n"/>
+    </row>
+    <row r="198">
+      <c r="M198" s="7" t="n"/>
+      <c r="N198" s="7" t="n"/>
+      <c r="O198" s="7" t="n"/>
+      <c r="P198" s="7" t="n"/>
+    </row>
+    <row r="199">
+      <c r="M199" s="7" t="n"/>
+      <c r="N199" s="7" t="n"/>
+      <c r="O199" s="7" t="n"/>
+      <c r="P199" s="7" t="n"/>
+    </row>
+    <row r="200">
+      <c r="M200" s="7" t="n"/>
+      <c r="N200" s="7" t="n"/>
+      <c r="O200" s="7" t="n"/>
+      <c r="P200" s="7" t="n"/>
+    </row>
+    <row r="201">
+      <c r="M201" s="7" t="n"/>
+      <c r="N201" s="7" t="n"/>
+      <c r="O201" s="7" t="n"/>
+      <c r="P201" s="7" t="n"/>
+    </row>
+    <row r="202">
+      <c r="M202" s="7" t="n"/>
+      <c r="N202" s="7" t="n"/>
+      <c r="O202" s="7" t="n"/>
+      <c r="P202" s="7" t="n"/>
+    </row>
+    <row r="203">
+      <c r="M203" s="7" t="n"/>
+      <c r="N203" s="7" t="n"/>
+      <c r="O203" s="7" t="n"/>
+      <c r="P203" s="7" t="n"/>
+    </row>
+    <row r="204">
+      <c r="M204" s="7" t="n"/>
+      <c r="N204" s="7" t="n"/>
+      <c r="O204" s="7" t="n"/>
+      <c r="P204" s="7" t="n"/>
+    </row>
+    <row r="205">
+      <c r="M205" s="7" t="n"/>
+      <c r="N205" s="7" t="n"/>
+      <c r="O205" s="7" t="n"/>
+      <c r="P205" s="7" t="n"/>
+    </row>
+    <row r="206">
+      <c r="M206" s="7" t="n"/>
+      <c r="N206" s="7" t="n"/>
+      <c r="O206" s="7" t="n"/>
+      <c r="P206" s="7" t="n"/>
+    </row>
+    <row r="207">
+      <c r="M207" s="7" t="n"/>
+      <c r="N207" s="7" t="n"/>
+      <c r="O207" s="7" t="n"/>
+      <c r="P207" s="7" t="n"/>
+    </row>
+    <row r="208">
+      <c r="M208" s="7" t="n"/>
+      <c r="N208" s="7" t="n"/>
+      <c r="O208" s="7" t="n"/>
+      <c r="P208" s="7" t="n"/>
+    </row>
+    <row r="209">
+      <c r="M209" s="7" t="n"/>
+      <c r="N209" s="7" t="n"/>
+      <c r="O209" s="7" t="n"/>
+      <c r="P209" s="7" t="n"/>
+    </row>
+    <row r="210">
+      <c r="M210" s="7" t="n"/>
+      <c r="N210" s="7" t="n"/>
+      <c r="O210" s="7" t="n"/>
+      <c r="P210" s="7" t="n"/>
+    </row>
+    <row r="211">
+      <c r="M211" s="7" t="n"/>
+      <c r="N211" s="7" t="n"/>
+      <c r="O211" s="7" t="n"/>
+      <c r="P211" s="7" t="n"/>
+    </row>
+    <row r="212">
+      <c r="M212" s="7" t="n"/>
+      <c r="N212" s="7" t="n"/>
+      <c r="O212" s="7" t="n"/>
+      <c r="P212" s="7" t="n"/>
+    </row>
+    <row r="213">
+      <c r="M213" s="7" t="n"/>
+      <c r="N213" s="7" t="n"/>
+      <c r="O213" s="7" t="n"/>
+      <c r="P213" s="7" t="n"/>
+    </row>
+    <row r="214">
+      <c r="M214" s="7" t="n"/>
+      <c r="N214" s="7" t="n"/>
+      <c r="O214" s="7" t="n"/>
+      <c r="P214" s="7" t="n"/>
+    </row>
+    <row r="215">
+      <c r="M215" s="7" t="n"/>
+      <c r="N215" s="7" t="n"/>
+      <c r="O215" s="7" t="n"/>
+      <c r="P215" s="7" t="n"/>
+    </row>
+    <row r="216">
+      <c r="M216" s="7" t="n"/>
+      <c r="N216" s="7" t="n"/>
+      <c r="O216" s="7" t="n"/>
+      <c r="P216" s="7" t="n"/>
+    </row>
+    <row r="217">
+      <c r="M217" s="7" t="n"/>
+      <c r="N217" s="7" t="n"/>
+      <c r="O217" s="7" t="n"/>
+      <c r="P217" s="7" t="n"/>
+    </row>
+    <row r="218">
+      <c r="M218" s="7" t="n"/>
+      <c r="N218" s="7" t="n"/>
+      <c r="O218" s="7" t="n"/>
+      <c r="P218" s="7" t="n"/>
+    </row>
+    <row r="219">
+      <c r="M219" s="7" t="n"/>
+      <c r="N219" s="7" t="n"/>
+      <c r="O219" s="7" t="n"/>
+      <c r="P219" s="7" t="n"/>
+    </row>
+    <row r="220">
+      <c r="M220" s="7" t="n"/>
+      <c r="N220" s="7" t="n"/>
+      <c r="O220" s="7" t="n"/>
+      <c r="P220" s="7" t="n"/>
+    </row>
+    <row r="221">
+      <c r="M221" s="7" t="n"/>
+      <c r="N221" s="7" t="n"/>
+      <c r="O221" s="7" t="n"/>
+      <c r="P221" s="7" t="n"/>
+    </row>
+    <row r="222">
+      <c r="M222" s="7" t="n"/>
+      <c r="N222" s="7" t="n"/>
+      <c r="O222" s="7" t="n"/>
+      <c r="P222" s="7" t="n"/>
+    </row>
+    <row r="223">
+      <c r="M223" s="7" t="n"/>
+      <c r="N223" s="7" t="n"/>
+      <c r="O223" s="7" t="n"/>
+      <c r="P223" s="7" t="n"/>
+    </row>
+    <row r="224">
+      <c r="M224" s="7" t="n"/>
+      <c r="N224" s="7" t="n"/>
+      <c r="O224" s="7" t="n"/>
+      <c r="P224" s="7" t="n"/>
+    </row>
+    <row r="225">
+      <c r="M225" s="7" t="n"/>
+      <c r="N225" s="7" t="n"/>
+      <c r="O225" s="7" t="n"/>
+      <c r="P225" s="7" t="n"/>
+    </row>
+    <row r="226">
+      <c r="M226" s="7" t="n"/>
+      <c r="N226" s="7" t="n"/>
+      <c r="O226" s="7" t="n"/>
+      <c r="P226" s="7" t="n"/>
+    </row>
+    <row r="227">
+      <c r="M227" s="7" t="n"/>
+      <c r="N227" s="7" t="n"/>
+      <c r="O227" s="7" t="n"/>
+      <c r="P227" s="7" t="n"/>
+    </row>
+    <row r="228">
+      <c r="M228" s="7" t="n"/>
+      <c r="N228" s="7" t="n"/>
+      <c r="O228" s="7" t="n"/>
+      <c r="P228" s="7" t="n"/>
+    </row>
+    <row r="229">
+      <c r="M229" s="7" t="n"/>
+      <c r="N229" s="7" t="n"/>
+      <c r="O229" s="7" t="n"/>
+      <c r="P229" s="7" t="n"/>
+    </row>
+    <row r="230">
+      <c r="M230" s="7" t="n"/>
+      <c r="N230" s="7" t="n"/>
+      <c r="O230" s="7" t="n"/>
+      <c r="P230" s="7" t="n"/>
+    </row>
+    <row r="231">
+      <c r="M231" s="7" t="n"/>
+      <c r="N231" s="7" t="n"/>
+      <c r="O231" s="7" t="n"/>
+      <c r="P231" s="7" t="n"/>
+    </row>
+    <row r="232">
+      <c r="M232" s="7" t="n"/>
+      <c r="N232" s="7" t="n"/>
+      <c r="O232" s="7" t="n"/>
+      <c r="P232" s="7" t="n"/>
+    </row>
+    <row r="233">
+      <c r="M233" s="7" t="n"/>
+      <c r="N233" s="7" t="n"/>
+      <c r="O233" s="7" t="n"/>
+      <c r="P233" s="7" t="n"/>
+    </row>
+    <row r="234">
+      <c r="M234" s="7" t="n"/>
+      <c r="N234" s="7" t="n"/>
+      <c r="O234" s="7" t="n"/>
+      <c r="P234" s="7" t="n"/>
+    </row>
+    <row r="235">
+      <c r="M235" s="7" t="n"/>
+      <c r="N235" s="7" t="n"/>
+      <c r="O235" s="7" t="n"/>
+      <c r="P235" s="7" t="n"/>
+    </row>
+    <row r="236">
+      <c r="M236" s="7" t="n"/>
+      <c r="N236" s="7" t="n"/>
+      <c r="O236" s="7" t="n"/>
+      <c r="P236" s="7" t="n"/>
+    </row>
+    <row r="237">
+      <c r="M237" s="7" t="n"/>
+      <c r="N237" s="7" t="n"/>
+      <c r="O237" s="7" t="n"/>
+      <c r="P237" s="7" t="n"/>
+    </row>
+    <row r="238">
+      <c r="M238" s="7" t="n"/>
+      <c r="N238" s="7" t="n"/>
+      <c r="O238" s="7" t="n"/>
+      <c r="P238" s="7" t="n"/>
+    </row>
+    <row r="239">
+      <c r="M239" s="7" t="n"/>
+      <c r="N239" s="7" t="n"/>
+      <c r="O239" s="7" t="n"/>
+      <c r="P239" s="7" t="n"/>
+    </row>
+    <row r="240">
+      <c r="M240" s="7" t="n"/>
+      <c r="N240" s="7" t="n"/>
+      <c r="O240" s="7" t="n"/>
+      <c r="P240" s="7" t="n"/>
+    </row>
+    <row r="241">
+      <c r="M241" s="7" t="n"/>
+      <c r="N241" s="7" t="n"/>
+      <c r="O241" s="7" t="n"/>
+      <c r="P241" s="7" t="n"/>
+    </row>
+    <row r="242">
+      <c r="M242" s="7" t="n"/>
+      <c r="N242" s="7" t="n"/>
+      <c r="O242" s="7" t="n"/>
+      <c r="P242" s="7" t="n"/>
+    </row>
+    <row r="243">
+      <c r="M243" s="7" t="n"/>
+      <c r="N243" s="7" t="n"/>
+      <c r="O243" s="7" t="n"/>
+      <c r="P243" s="7" t="n"/>
+    </row>
+    <row r="244">
+      <c r="M244" s="7" t="n"/>
+      <c r="N244" s="7" t="n"/>
+      <c r="O244" s="7" t="n"/>
+      <c r="P244" s="7" t="n"/>
+    </row>
+    <row r="245">
+      <c r="M245" s="7" t="n"/>
+      <c r="N245" s="7" t="n"/>
+      <c r="O245" s="7" t="n"/>
+      <c r="P245" s="7" t="n"/>
+    </row>
+    <row r="246">
+      <c r="M246" s="7" t="n"/>
+      <c r="N246" s="7" t="n"/>
+      <c r="O246" s="7" t="n"/>
+      <c r="P246" s="7" t="n"/>
+    </row>
+    <row r="247">
+      <c r="M247" s="7" t="n"/>
+      <c r="N247" s="7" t="n"/>
+      <c r="O247" s="7" t="n"/>
+      <c r="P247" s="7" t="n"/>
+    </row>
+    <row r="248">
+      <c r="M248" s="7" t="n"/>
+      <c r="N248" s="7" t="n"/>
+      <c r="O248" s="7" t="n"/>
+      <c r="P248" s="7" t="n"/>
+    </row>
+    <row r="249">
+      <c r="M249" s="7" t="n"/>
+      <c r="N249" s="7" t="n"/>
+      <c r="O249" s="7" t="n"/>
+      <c r="P249" s="7" t="n"/>
+    </row>
+    <row r="250">
+      <c r="M250" s="7" t="n"/>
+      <c r="N250" s="7" t="n"/>
+      <c r="O250" s="7" t="n"/>
+      <c r="P250" s="7" t="n"/>
+    </row>
+    <row r="251">
+      <c r="M251" s="7" t="n"/>
+      <c r="N251" s="7" t="n"/>
+      <c r="O251" s="7" t="n"/>
+      <c r="P251" s="7" t="n"/>
+    </row>
+    <row r="252">
+      <c r="M252" s="7" t="n"/>
+      <c r="N252" s="7" t="n"/>
+      <c r="O252" s="7" t="n"/>
+      <c r="P252" s="7" t="n"/>
+    </row>
+    <row r="253">
+      <c r="M253" s="7" t="n"/>
+      <c r="N253" s="7" t="n"/>
+      <c r="O253" s="7" t="n"/>
+      <c r="P253" s="7" t="n"/>
+    </row>
+    <row r="254">
+      <c r="M254" s="7" t="n"/>
+      <c r="N254" s="7" t="n"/>
+      <c r="O254" s="7" t="n"/>
+      <c r="P254" s="7" t="n"/>
+    </row>
+    <row r="255">
+      <c r="M255" s="7" t="n"/>
+      <c r="N255" s="7" t="n"/>
+      <c r="O255" s="7" t="n"/>
+      <c r="P255" s="7" t="n"/>
+    </row>
+    <row r="256">
+      <c r="M256" s="7" t="n"/>
+      <c r="N256" s="7" t="n"/>
+      <c r="O256" s="7" t="n"/>
+      <c r="P256" s="7" t="n"/>
+    </row>
+    <row r="257">
+      <c r="M257" s="7" t="n"/>
+      <c r="N257" s="7" t="n"/>
+      <c r="O257" s="7" t="n"/>
+      <c r="P257" s="7" t="n"/>
+    </row>
+    <row r="258">
+      <c r="M258" s="7" t="n"/>
+      <c r="N258" s="7" t="n"/>
+      <c r="O258" s="7" t="n"/>
+      <c r="P258" s="7" t="n"/>
+    </row>
+    <row r="259">
+      <c r="M259" s="7" t="n"/>
+      <c r="N259" s="7" t="n"/>
+      <c r="O259" s="7" t="n"/>
+      <c r="P259" s="7" t="n"/>
+    </row>
+    <row r="260">
+      <c r="M260" s="7" t="n"/>
+      <c r="N260" s="7" t="n"/>
+      <c r="O260" s="7" t="n"/>
+      <c r="P260" s="7" t="n"/>
+    </row>
+    <row r="261">
+      <c r="M261" s="7" t="n"/>
+      <c r="N261" s="7" t="n"/>
+      <c r="O261" s="7" t="n"/>
+      <c r="P261" s="7" t="n"/>
+    </row>
+    <row r="262">
+      <c r="M262" s="7" t="n"/>
+      <c r="N262" s="7" t="n"/>
+      <c r="O262" s="7" t="n"/>
+      <c r="P262" s="7" t="n"/>
+    </row>
+    <row r="263">
+      <c r="M263" s="7" t="n"/>
+      <c r="N263" s="7" t="n"/>
+      <c r="O263" s="7" t="n"/>
+      <c r="P263" s="7" t="n"/>
+    </row>
+    <row r="264">
+      <c r="M264" s="7" t="n"/>
+      <c r="N264" s="7" t="n"/>
+      <c r="O264" s="7" t="n"/>
+      <c r="P264" s="7" t="n"/>
+    </row>
+    <row r="265">
+      <c r="M265" s="7" t="n"/>
+      <c r="N265" s="7" t="n"/>
+      <c r="O265" s="7" t="n"/>
+      <c r="P265" s="7" t="n"/>
+    </row>
+    <row r="266">
+      <c r="M266" s="7" t="n"/>
+      <c r="N266" s="7" t="n"/>
+      <c r="O266" s="7" t="n"/>
+      <c r="P266" s="7" t="n"/>
+    </row>
+    <row r="267">
+      <c r="M267" s="7" t="n"/>
+      <c r="N267" s="7" t="n"/>
+      <c r="O267" s="7" t="n"/>
+      <c r="P267" s="7" t="n"/>
+    </row>
+    <row r="268">
+      <c r="M268" s="7" t="n"/>
+      <c r="N268" s="7" t="n"/>
+      <c r="O268" s="7" t="n"/>
+      <c r="P268" s="7" t="n"/>
+    </row>
+    <row r="269">
+      <c r="M269" s="7" t="n"/>
+      <c r="N269" s="7" t="n"/>
+      <c r="O269" s="7" t="n"/>
+      <c r="P269" s="7" t="n"/>
+    </row>
+    <row r="270">
+      <c r="M270" s="7" t="n"/>
+      <c r="N270" s="7" t="n"/>
+      <c r="O270" s="7" t="n"/>
+      <c r="P270" s="7" t="n"/>
+    </row>
+    <row r="271">
+      <c r="M271" s="7" t="n"/>
+      <c r="N271" s="7" t="n"/>
+      <c r="O271" s="7" t="n"/>
+      <c r="P271" s="7" t="n"/>
+    </row>
+    <row r="272">
+      <c r="M272" s="7" t="n"/>
+      <c r="N272" s="7" t="n"/>
+      <c r="O272" s="7" t="n"/>
+      <c r="P272" s="7" t="n"/>
+    </row>
+    <row r="273">
+      <c r="M273" s="7" t="n"/>
+      <c r="N273" s="7" t="n"/>
+      <c r="O273" s="7" t="n"/>
+      <c r="P273" s="7" t="n"/>
+    </row>
+    <row r="274">
+      <c r="M274" s="7" t="n"/>
+      <c r="N274" s="7" t="n"/>
+      <c r="O274" s="7" t="n"/>
+      <c r="P274" s="7" t="n"/>
+    </row>
+    <row r="275">
+      <c r="M275" s="7" t="n"/>
+      <c r="N275" s="7" t="n"/>
+      <c r="O275" s="7" t="n"/>
+      <c r="P275" s="7" t="n"/>
+    </row>
+    <row r="276">
+      <c r="M276" s="7" t="n"/>
+      <c r="N276" s="7" t="n"/>
+      <c r="O276" s="7" t="n"/>
+      <c r="P276" s="7" t="n"/>
+    </row>
+    <row r="277">
+      <c r="M277" s="7" t="n"/>
+      <c r="N277" s="7" t="n"/>
+      <c r="O277" s="7" t="n"/>
+      <c r="P277" s="7" t="n"/>
+    </row>
+    <row r="278">
+      <c r="M278" s="7" t="n"/>
+      <c r="N278" s="7" t="n"/>
+      <c r="O278" s="7" t="n"/>
+      <c r="P278" s="7" t="n"/>
+    </row>
+    <row r="279">
+      <c r="M279" s="7" t="n"/>
+      <c r="N279" s="7" t="n"/>
+      <c r="O279" s="7" t="n"/>
+      <c r="P279" s="7" t="n"/>
+    </row>
+    <row r="280">
+      <c r="M280" s="7" t="n"/>
+      <c r="N280" s="7" t="n"/>
+      <c r="O280" s="7" t="n"/>
+      <c r="P280" s="7" t="n"/>
+    </row>
+    <row r="281">
+      <c r="M281" s="7" t="n"/>
+      <c r="N281" s="7" t="n"/>
+      <c r="O281" s="7" t="n"/>
+      <c r="P281" s="7" t="n"/>
+    </row>
+    <row r="282">
+      <c r="M282" s="7" t="n"/>
+      <c r="N282" s="7" t="n"/>
+      <c r="O282" s="7" t="n"/>
+      <c r="P282" s="7" t="n"/>
+    </row>
+    <row r="283">
+      <c r="M283" s="7" t="n"/>
+      <c r="N283" s="7" t="n"/>
+      <c r="O283" s="7" t="n"/>
+      <c r="P283" s="7" t="n"/>
+    </row>
+    <row r="284">
+      <c r="M284" s="7" t="n"/>
+      <c r="N284" s="7" t="n"/>
+      <c r="O284" s="7" t="n"/>
+      <c r="P284" s="7" t="n"/>
+    </row>
+    <row r="285">
+      <c r="M285" s="7" t="n"/>
+      <c r="N285" s="7" t="n"/>
+      <c r="O285" s="7" t="n"/>
+      <c r="P285" s="7" t="n"/>
+    </row>
+    <row r="286">
+      <c r="M286" s="7" t="n"/>
+      <c r="N286" s="7" t="n"/>
+      <c r="O286" s="7" t="n"/>
+      <c r="P286" s="7" t="n"/>
+    </row>
+    <row r="287">
+      <c r="M287" s="7" t="n"/>
+      <c r="N287" s="7" t="n"/>
+      <c r="O287" s="7" t="n"/>
+      <c r="P287" s="7" t="n"/>
+    </row>
+    <row r="288">
+      <c r="M288" s="7" t="n"/>
+      <c r="N288" s="7" t="n"/>
+      <c r="O288" s="7" t="n"/>
+      <c r="P288" s="7" t="n"/>
+    </row>
+    <row r="289">
+      <c r="M289" s="7" t="n"/>
+      <c r="N289" s="7" t="n"/>
+      <c r="O289" s="7" t="n"/>
+      <c r="P289" s="7" t="n"/>
+    </row>
+    <row r="290">
+      <c r="M290" s="7" t="n"/>
+      <c r="N290" s="7" t="n"/>
+      <c r="O290" s="7" t="n"/>
+      <c r="P290" s="7" t="n"/>
+    </row>
+    <row r="291">
+      <c r="M291" s="7" t="n"/>
+      <c r="N291" s="7" t="n"/>
+      <c r="O291" s="7" t="n"/>
+      <c r="P291" s="7" t="n"/>
+    </row>
+    <row r="292">
+      <c r="M292" s="7" t="n"/>
+      <c r="N292" s="7" t="n"/>
+      <c r="O292" s="7" t="n"/>
+      <c r="P292" s="7" t="n"/>
+    </row>
+    <row r="293">
+      <c r="M293" s="7" t="n"/>
+      <c r="N293" s="7" t="n"/>
+      <c r="O293" s="7" t="n"/>
+      <c r="P293" s="7" t="n"/>
+    </row>
+    <row r="294">
+      <c r="M294" s="7" t="n"/>
+      <c r="N294" s="7" t="n"/>
+      <c r="O294" s="7" t="n"/>
+      <c r="P294" s="7" t="n"/>
+    </row>
+    <row r="295">
+      <c r="M295" s="7" t="n"/>
+      <c r="N295" s="7" t="n"/>
+      <c r="O295" s="7" t="n"/>
+      <c r="P295" s="7" t="n"/>
+    </row>
+    <row r="296">
+      <c r="M296" s="7" t="n"/>
+      <c r="N296" s="7" t="n"/>
+      <c r="O296" s="7" t="n"/>
+      <c r="P296" s="7" t="n"/>
+    </row>
+    <row r="297">
+      <c r="M297" s="7" t="n"/>
+      <c r="N297" s="7" t="n"/>
+      <c r="O297" s="7" t="n"/>
+      <c r="P297" s="7" t="n"/>
+    </row>
+    <row r="298">
+      <c r="M298" s="7" t="n"/>
+      <c r="N298" s="7" t="n"/>
+      <c r="O298" s="7" t="n"/>
+      <c r="P298" s="7" t="n"/>
+    </row>
+    <row r="299">
+      <c r="M299" s="7" t="n"/>
+      <c r="N299" s="7" t="n"/>
+      <c r="O299" s="7" t="n"/>
+      <c r="P299" s="7" t="n"/>
+    </row>
+    <row r="300">
+      <c r="M300" s="7" t="n"/>
+      <c r="N300" s="7" t="n"/>
+      <c r="O300" s="7" t="n"/>
+      <c r="P300" s="7" t="n"/>
+    </row>
+    <row r="301">
+      <c r="M301" s="7" t="n"/>
+      <c r="N301" s="7" t="n"/>
+      <c r="O301" s="7" t="n"/>
+      <c r="P301" s="7" t="n"/>
+    </row>
+    <row r="302">
+      <c r="M302" s="7" t="n"/>
+      <c r="N302" s="7" t="n"/>
+      <c r="O302" s="7" t="n"/>
+      <c r="P302" s="7" t="n"/>
+    </row>
+    <row r="303">
+      <c r="M303" s="7" t="n"/>
+      <c r="N303" s="7" t="n"/>
+      <c r="O303" s="7" t="n"/>
+      <c r="P303" s="7" t="n"/>
+    </row>
+    <row r="304">
+      <c r="M304" s="7" t="n"/>
+      <c r="N304" s="7" t="n"/>
+      <c r="O304" s="7" t="n"/>
+      <c r="P304" s="7" t="n"/>
+    </row>
+    <row r="305">
+      <c r="M305" s="7" t="n"/>
+      <c r="N305" s="7" t="n"/>
+      <c r="O305" s="7" t="n"/>
+      <c r="P305" s="7" t="n"/>
+    </row>
+    <row r="306">
+      <c r="M306" s="7" t="n"/>
+      <c r="N306" s="7" t="n"/>
+      <c r="O306" s="7" t="n"/>
+      <c r="P306" s="7" t="n"/>
+    </row>
+    <row r="307">
+      <c r="M307" s="7" t="n"/>
+      <c r="N307" s="7" t="n"/>
+      <c r="O307" s="7" t="n"/>
+      <c r="P307" s="7" t="n"/>
+    </row>
+    <row r="308">
+      <c r="M308" s="7" t="n"/>
+      <c r="N308" s="7" t="n"/>
+      <c r="O308" s="7" t="n"/>
+      <c r="P308" s="7" t="n"/>
+    </row>
+    <row r="309">
+      <c r="M309" s="7" t="n"/>
+      <c r="N309" s="7" t="n"/>
+      <c r="O309" s="7" t="n"/>
+      <c r="P309" s="7" t="n"/>
+    </row>
+    <row r="310">
+      <c r="M310" s="7" t="n"/>
+      <c r="N310" s="7" t="n"/>
+      <c r="O310" s="7" t="n"/>
+      <c r="P310" s="7" t="n"/>
+    </row>
+    <row r="311">
+      <c r="M311" s="7" t="n"/>
+      <c r="N311" s="7" t="n"/>
+      <c r="O311" s="7" t="n"/>
+      <c r="P311" s="7" t="n"/>
+    </row>
+    <row r="312">
+      <c r="M312" s="7" t="n"/>
+      <c r="N312" s="7" t="n"/>
+      <c r="O312" s="7" t="n"/>
+      <c r="P312" s="7" t="n"/>
+    </row>
+    <row r="313">
+      <c r="M313" s="7" t="n"/>
+      <c r="N313" s="7" t="n"/>
+      <c r="O313" s="7" t="n"/>
+      <c r="P313" s="7" t="n"/>
+    </row>
+    <row r="314">
+      <c r="M314" s="7" t="n"/>
+      <c r="N314" s="7" t="n"/>
+      <c r="O314" s="7" t="n"/>
+      <c r="P314" s="7" t="n"/>
+    </row>
+    <row r="315">
+      <c r="M315" s="7" t="n"/>
+      <c r="N315" s="7" t="n"/>
+      <c r="O315" s="7" t="n"/>
+      <c r="P315" s="7" t="n"/>
+    </row>
+    <row r="316">
+      <c r="M316" s="7" t="n"/>
+      <c r="N316" s="7" t="n"/>
+      <c r="O316" s="7" t="n"/>
+      <c r="P316" s="7" t="n"/>
+    </row>
+    <row r="317">
+      <c r="M317" s="7" t="n"/>
+      <c r="N317" s="7" t="n"/>
+      <c r="O317" s="7" t="n"/>
+      <c r="P317" s="7" t="n"/>
+    </row>
+    <row r="318">
+      <c r="M318" s="7" t="n"/>
+      <c r="N318" s="7" t="n"/>
+      <c r="O318" s="7" t="n"/>
+      <c r="P318" s="7" t="n"/>
+    </row>
+    <row r="319">
+      <c r="M319" s="7" t="n"/>
+      <c r="N319" s="7" t="n"/>
+      <c r="O319" s="7" t="n"/>
+      <c r="P319" s="7" t="n"/>
+    </row>
+    <row r="320">
+      <c r="M320" s="7" t="n"/>
+      <c r="N320" s="7" t="n"/>
+      <c r="O320" s="7" t="n"/>
+      <c r="P320" s="7" t="n"/>
+    </row>
+    <row r="321">
+      <c r="M321" s="7" t="n"/>
+      <c r="N321" s="7" t="n"/>
+      <c r="O321" s="7" t="n"/>
+      <c r="P321" s="7" t="n"/>
+    </row>
+    <row r="322">
+      <c r="M322" s="7" t="n"/>
+      <c r="N322" s="7" t="n"/>
+      <c r="O322" s="7" t="n"/>
+      <c r="P322" s="7" t="n"/>
+    </row>
+    <row r="323">
+      <c r="M323" s="7" t="n"/>
+      <c r="N323" s="7" t="n"/>
+      <c r="O323" s="7" t="n"/>
+      <c r="P323" s="7" t="n"/>
+    </row>
+    <row r="324">
+      <c r="M324" s="7" t="n"/>
+      <c r="N324" s="7" t="n"/>
+      <c r="O324" s="7" t="n"/>
+      <c r="P324" s="7" t="n"/>
+    </row>
+    <row r="325">
+      <c r="M325" s="7" t="n"/>
+      <c r="N325" s="7" t="n"/>
+      <c r="O325" s="7" t="n"/>
+      <c r="P325" s="7" t="n"/>
+    </row>
+    <row r="326">
+      <c r="M326" s="7" t="n"/>
+      <c r="N326" s="7" t="n"/>
+      <c r="O326" s="7" t="n"/>
+      <c r="P326" s="7" t="n"/>
+    </row>
+    <row r="327">
+      <c r="M327" s="7" t="n"/>
+      <c r="N327" s="7" t="n"/>
+      <c r="O327" s="7" t="n"/>
+      <c r="P327" s="7" t="n"/>
+    </row>
+    <row r="328">
+      <c r="M328" s="7" t="n"/>
+      <c r="N328" s="7" t="n"/>
+      <c r="O328" s="7" t="n"/>
+      <c r="P328" s="7" t="n"/>
+    </row>
+    <row r="329">
+      <c r="M329" s="7" t="n"/>
+      <c r="N329" s="7" t="n"/>
+      <c r="O329" s="7" t="n"/>
+      <c r="P329" s="7" t="n"/>
+    </row>
+    <row r="330">
+      <c r="M330" s="7" t="n"/>
+      <c r="N330" s="7" t="n"/>
+      <c r="O330" s="7" t="n"/>
+      <c r="P330" s="7" t="n"/>
+    </row>
+    <row r="331">
+      <c r="M331" s="7" t="n"/>
+      <c r="N331" s="7" t="n"/>
+      <c r="O331" s="7" t="n"/>
+      <c r="P331" s="7" t="n"/>
+    </row>
+    <row r="332">
+      <c r="M332" s="7" t="n"/>
+      <c r="N332" s="7" t="n"/>
+      <c r="O332" s="7" t="n"/>
+      <c r="P332" s="7" t="n"/>
+    </row>
+    <row r="333">
+      <c r="M333" s="7" t="n"/>
+      <c r="N333" s="7" t="n"/>
+      <c r="O333" s="7" t="n"/>
+      <c r="P333" s="7" t="n"/>
+    </row>
+    <row r="334">
+      <c r="M334" s="7" t="n"/>
+      <c r="N334" s="7" t="n"/>
+      <c r="O334" s="7" t="n"/>
+      <c r="P334" s="7" t="n"/>
+    </row>
+    <row r="335">
+      <c r="M335" s="7" t="n"/>
+      <c r="N335" s="7" t="n"/>
+      <c r="O335" s="7" t="n"/>
+      <c r="P335" s="7" t="n"/>
+    </row>
+    <row r="336">
+      <c r="M336" s="7" t="n"/>
+      <c r="N336" s="7" t="n"/>
+      <c r="O336" s="7" t="n"/>
+      <c r="P336" s="7" t="n"/>
+    </row>
+    <row r="337">
+      <c r="M337" s="7" t="n"/>
+      <c r="N337" s="7" t="n"/>
+      <c r="O337" s="7" t="n"/>
+      <c r="P337" s="7" t="n"/>
+    </row>
+    <row r="338">
+      <c r="M338" s="7" t="n"/>
+      <c r="N338" s="7" t="n"/>
+      <c r="O338" s="7" t="n"/>
+      <c r="P338" s="7" t="n"/>
+    </row>
+    <row r="339">
+      <c r="M339" s="7" t="n"/>
+      <c r="N339" s="7" t="n"/>
+      <c r="O339" s="7" t="n"/>
+      <c r="P339" s="7" t="n"/>
+    </row>
+    <row r="340">
+      <c r="M340" s="7" t="n"/>
+      <c r="N340" s="7" t="n"/>
+      <c r="O340" s="7" t="n"/>
+      <c r="P340" s="7" t="n"/>
+    </row>
+    <row r="341">
+      <c r="M341" s="7" t="n"/>
+      <c r="N341" s="7" t="n"/>
+      <c r="O341" s="7" t="n"/>
+      <c r="P341" s="7" t="n"/>
+    </row>
+    <row r="342">
+      <c r="M342" s="7" t="n"/>
+      <c r="N342" s="7" t="n"/>
+      <c r="O342" s="7" t="n"/>
+      <c r="P342" s="7" t="n"/>
+    </row>
+    <row r="343">
+      <c r="M343" s="7" t="n"/>
+      <c r="N343" s="7" t="n"/>
+      <c r="O343" s="7" t="n"/>
+      <c r="P343" s="7" t="n"/>
+    </row>
+    <row r="344">
+      <c r="M344" s="7" t="n"/>
+      <c r="N344" s="7" t="n"/>
+      <c r="O344" s="7" t="n"/>
+      <c r="P344" s="7" t="n"/>
+    </row>
+    <row r="345">
+      <c r="M345" s="7" t="n"/>
+      <c r="N345" s="7" t="n"/>
+      <c r="O345" s="7" t="n"/>
+      <c r="P345" s="7" t="n"/>
+    </row>
+    <row r="346">
+      <c r="M346" s="7" t="n"/>
+      <c r="N346" s="7" t="n"/>
+      <c r="O346" s="7" t="n"/>
+      <c r="P346" s="7" t="n"/>
+    </row>
+    <row r="347">
+      <c r="M347" s="7" t="n"/>
+      <c r="N347" s="7" t="n"/>
+      <c r="O347" s="7" t="n"/>
+      <c r="P347" s="7" t="n"/>
+    </row>
+    <row r="348">
+      <c r="M348" s="7" t="n"/>
+      <c r="N348" s="7" t="n"/>
+      <c r="O348" s="7" t="n"/>
+      <c r="P348" s="7" t="n"/>
+    </row>
+    <row r="349">
+      <c r="M349" s="7" t="n"/>
+      <c r="N349" s="7" t="n"/>
+      <c r="O349" s="7" t="n"/>
+      <c r="P349" s="7" t="n"/>
+    </row>
+    <row r="350">
+      <c r="M350" s="7" t="n"/>
+      <c r="N350" s="7" t="n"/>
+      <c r="O350" s="7" t="n"/>
+      <c r="P350" s="7" t="n"/>
+    </row>
+    <row r="351">
+      <c r="M351" s="7" t="n"/>
+      <c r="N351" s="7" t="n"/>
+      <c r="O351" s="7" t="n"/>
+      <c r="P351" s="7" t="n"/>
+    </row>
+    <row r="352">
+      <c r="M352" s="7" t="n"/>
+      <c r="N352" s="7" t="n"/>
+      <c r="O352" s="7" t="n"/>
+      <c r="P352" s="7" t="n"/>
+    </row>
+    <row r="353">
+      <c r="M353" s="7" t="n"/>
+      <c r="N353" s="7" t="n"/>
+      <c r="O353" s="7" t="n"/>
+      <c r="P353" s="7" t="n"/>
+    </row>
+    <row r="354">
+      <c r="M354" s="7" t="n"/>
+      <c r="N354" s="7" t="n"/>
+      <c r="O354" s="7" t="n"/>
+      <c r="P354" s="7" t="n"/>
+    </row>
+    <row r="355">
+      <c r="M355" s="7" t="n"/>
+      <c r="N355" s="7" t="n"/>
+      <c r="O355" s="7" t="n"/>
+      <c r="P355" s="7" t="n"/>
+    </row>
+    <row r="356">
+      <c r="M356" s="7" t="n"/>
+      <c r="N356" s="7" t="n"/>
+      <c r="O356" s="7" t="n"/>
+      <c r="P356" s="7" t="n"/>
+    </row>
+    <row r="357">
+      <c r="M357" s="7" t="n"/>
+      <c r="N357" s="7" t="n"/>
+      <c r="O357" s="7" t="n"/>
+      <c r="P357" s="7" t="n"/>
+    </row>
+    <row r="358">
+      <c r="M358" s="7" t="n"/>
+      <c r="N358" s="7" t="n"/>
+      <c r="O358" s="7" t="n"/>
+      <c r="P358" s="7" t="n"/>
+    </row>
+    <row r="359">
+      <c r="M359" s="7" t="n"/>
+      <c r="N359" s="7" t="n"/>
+      <c r="O359" s="7" t="n"/>
+      <c r="P359" s="7" t="n"/>
+    </row>
+    <row r="360">
+      <c r="M360" s="7" t="n"/>
+      <c r="N360" s="7" t="n"/>
+      <c r="O360" s="7" t="n"/>
+      <c r="P360" s="7" t="n"/>
+    </row>
+    <row r="361">
+      <c r="M361" s="7" t="n"/>
+      <c r="N361" s="7" t="n"/>
+      <c r="O361" s="7" t="n"/>
+      <c r="P361" s="7" t="n"/>
+    </row>
+    <row r="362">
+      <c r="M362" s="7" t="n"/>
+      <c r="N362" s="7" t="n"/>
+      <c r="O362" s="7" t="n"/>
+      <c r="P362" s="7" t="n"/>
+    </row>
+    <row r="363">
+      <c r="M363" s="7" t="n"/>
+      <c r="N363" s="7" t="n"/>
+      <c r="O363" s="7" t="n"/>
+      <c r="P363" s="7" t="n"/>
+    </row>
+    <row r="364">
+      <c r="M364" s="7" t="n"/>
+      <c r="N364" s="7" t="n"/>
+      <c r="O364" s="7" t="n"/>
+      <c r="P364" s="7" t="n"/>
+    </row>
+    <row r="365">
+      <c r="M365" s="7" t="n"/>
+      <c r="N365" s="7" t="n"/>
+      <c r="O365" s="7" t="n"/>
+      <c r="P365" s="7" t="n"/>
+    </row>
+    <row r="366">
+      <c r="M366" s="7" t="n"/>
+      <c r="N366" s="7" t="n"/>
+      <c r="O366" s="7" t="n"/>
+      <c r="P366" s="7" t="n"/>
+    </row>
+    <row r="367">
+      <c r="M367" s="7" t="n"/>
+      <c r="N367" s="7" t="n"/>
+      <c r="O367" s="7" t="n"/>
+      <c r="P367" s="7" t="n"/>
+    </row>
+    <row r="368">
+      <c r="M368" s="7" t="n"/>
+      <c r="N368" s="7" t="n"/>
+      <c r="O368" s="7" t="n"/>
+      <c r="P368" s="7" t="n"/>
+    </row>
+    <row r="369">
+      <c r="M369" s="7" t="n"/>
+      <c r="N369" s="7" t="n"/>
+      <c r="O369" s="7" t="n"/>
+      <c r="P369" s="7" t="n"/>
+    </row>
+    <row r="370">
+      <c r="M370" s="7" t="n"/>
+      <c r="N370" s="7" t="n"/>
+      <c r="O370" s="7" t="n"/>
+      <c r="P370" s="7" t="n"/>
+    </row>
+    <row r="371">
+      <c r="M371" s="7" t="n"/>
+      <c r="N371" s="7" t="n"/>
+      <c r="O371" s="7" t="n"/>
+      <c r="P371" s="7" t="n"/>
+    </row>
+    <row r="372">
+      <c r="M372" s="7" t="n"/>
+      <c r="N372" s="7" t="n"/>
+      <c r="O372" s="7" t="n"/>
+      <c r="P372" s="7" t="n"/>
+    </row>
+    <row r="373">
+      <c r="M373" s="7" t="n"/>
+      <c r="N373" s="7" t="n"/>
+      <c r="O373" s="7" t="n"/>
+      <c r="P373" s="7" t="n"/>
+    </row>
+    <row r="374">
+      <c r="M374" s="7" t="n"/>
+      <c r="N374" s="7" t="n"/>
+      <c r="O374" s="7" t="n"/>
+      <c r="P374" s="7" t="n"/>
+    </row>
+    <row r="375">
+      <c r="M375" s="7" t="n"/>
+      <c r="N375" s="7" t="n"/>
+      <c r="O375" s="7" t="n"/>
+      <c r="P375" s="7" t="n"/>
+    </row>
+    <row r="376">
+      <c r="M376" s="7" t="n"/>
+      <c r="N376" s="7" t="n"/>
+      <c r="O376" s="7" t="n"/>
+      <c r="P376" s="7" t="n"/>
+    </row>
+    <row r="377">
+      <c r="M377" s="7" t="n"/>
+      <c r="N377" s="7" t="n"/>
+      <c r="O377" s="7" t="n"/>
+      <c r="P377" s="7" t="n"/>
+    </row>
+    <row r="378">
+      <c r="M378" s="7" t="n"/>
+      <c r="N378" s="7" t="n"/>
+      <c r="O378" s="7" t="n"/>
+      <c r="P378" s="7" t="n"/>
+    </row>
+    <row r="379">
+      <c r="M379" s="7" t="n"/>
+      <c r="N379" s="7" t="n"/>
+      <c r="O379" s="7" t="n"/>
+      <c r="P379" s="7" t="n"/>
+    </row>
+    <row r="380">
+      <c r="M380" s="7" t="n"/>
+      <c r="N380" s="7" t="n"/>
+      <c r="O380" s="7" t="n"/>
+      <c r="P380" s="7" t="n"/>
+    </row>
+    <row r="381">
+      <c r="M381" s="7" t="n"/>
+      <c r="N381" s="7" t="n"/>
+      <c r="O381" s="7" t="n"/>
+      <c r="P381" s="7" t="n"/>
+    </row>
+    <row r="382">
+      <c r="M382" s="7" t="n"/>
+      <c r="N382" s="7" t="n"/>
+      <c r="O382" s="7" t="n"/>
+      <c r="P382" s="7" t="n"/>
+    </row>
+    <row r="383">
+      <c r="M383" s="7" t="n"/>
+      <c r="N383" s="7" t="n"/>
+      <c r="O383" s="7" t="n"/>
+      <c r="P383" s="7" t="n"/>
+    </row>
+    <row r="384">
+      <c r="M384" s="7" t="n"/>
+      <c r="N384" s="7" t="n"/>
+      <c r="O384" s="7" t="n"/>
+      <c r="P384" s="7" t="n"/>
+    </row>
+    <row r="385">
+      <c r="M385" s="7" t="n"/>
+      <c r="N385" s="7" t="n"/>
+      <c r="O385" s="7" t="n"/>
+      <c r="P385" s="7" t="n"/>
+    </row>
+    <row r="386">
+      <c r="M386" s="7" t="n"/>
+      <c r="N386" s="7" t="n"/>
+      <c r="O386" s="7" t="n"/>
+      <c r="P386" s="7" t="n"/>
+    </row>
+    <row r="387">
+      <c r="M387" s="7" t="n"/>
+      <c r="N387" s="7" t="n"/>
+      <c r="O387" s="7" t="n"/>
+      <c r="P387" s="7" t="n"/>
+    </row>
+    <row r="388">
+      <c r="M388" s="7" t="n"/>
+      <c r="N388" s="7" t="n"/>
+      <c r="O388" s="7" t="n"/>
+      <c r="P388" s="7" t="n"/>
+    </row>
+    <row r="389">
+      <c r="M389" s="7" t="n"/>
+      <c r="N389" s="7" t="n"/>
+      <c r="O389" s="7" t="n"/>
+      <c r="P389" s="7" t="n"/>
+    </row>
+    <row r="390">
+      <c r="M390" s="7" t="n"/>
+      <c r="N390" s="7" t="n"/>
+      <c r="O390" s="7" t="n"/>
+      <c r="P390" s="7" t="n"/>
+    </row>
+    <row r="391">
+      <c r="M391" s="7" t="n"/>
+      <c r="N391" s="7" t="n"/>
+      <c r="O391" s="7" t="n"/>
+      <c r="P391" s="7" t="n"/>
+    </row>
+    <row r="392">
+      <c r="M392" s="7" t="n"/>
+      <c r="N392" s="7" t="n"/>
+      <c r="O392" s="7" t="n"/>
+      <c r="P392" s="7" t="n"/>
+    </row>
+    <row r="393">
+      <c r="M393" s="7" t="n"/>
+      <c r="N393" s="7" t="n"/>
+      <c r="O393" s="7" t="n"/>
+      <c r="P393" s="7" t="n"/>
+    </row>
+    <row r="394">
+      <c r="M394" s="7" t="n"/>
+      <c r="N394" s="7" t="n"/>
+      <c r="O394" s="7" t="n"/>
+      <c r="P394" s="7" t="n"/>
+    </row>
+    <row r="395">
+      <c r="M395" s="7" t="n"/>
+      <c r="N395" s="7" t="n"/>
+      <c r="O395" s="7" t="n"/>
+      <c r="P395" s="7" t="n"/>
+    </row>
+    <row r="396">
+      <c r="M396" s="7" t="n"/>
+      <c r="N396" s="7" t="n"/>
+      <c r="O396" s="7" t="n"/>
+      <c r="P396" s="7" t="n"/>
+    </row>
+    <row r="397">
+      <c r="M397" s="7" t="n"/>
+      <c r="N397" s="7" t="n"/>
+      <c r="O397" s="7" t="n"/>
+      <c r="P397" s="7" t="n"/>
+    </row>
+    <row r="398">
+      <c r="M398" s="7" t="n"/>
+      <c r="N398" s="7" t="n"/>
+      <c r="O398" s="7" t="n"/>
+      <c r="P398" s="7" t="n"/>
+    </row>
+    <row r="399">
+      <c r="M399" s="7" t="n"/>
+      <c r="N399" s="7" t="n"/>
+      <c r="O399" s="7" t="n"/>
+      <c r="P399" s="7" t="n"/>
+    </row>
+    <row r="400">
+      <c r="M400" s="7" t="n"/>
+      <c r="N400" s="7" t="n"/>
+      <c r="O400" s="7" t="n"/>
+      <c r="P400" s="7" t="n"/>
+    </row>
+    <row r="401">
+      <c r="M401" s="7" t="n"/>
+      <c r="N401" s="7" t="n"/>
+      <c r="O401" s="7" t="n"/>
+      <c r="P401" s="7" t="n"/>
+    </row>
+    <row r="402">
+      <c r="M402" s="7" t="n"/>
+      <c r="N402" s="7" t="n"/>
+      <c r="O402" s="7" t="n"/>
+      <c r="P402" s="7" t="n"/>
+    </row>
+    <row r="403">
+      <c r="M403" s="7" t="n"/>
+      <c r="N403" s="7" t="n"/>
+      <c r="O403" s="7" t="n"/>
+      <c r="P403" s="7" t="n"/>
+    </row>
+    <row r="404">
+      <c r="M404" s="7" t="n"/>
+      <c r="N404" s="7" t="n"/>
+      <c r="O404" s="7" t="n"/>
+      <c r="P404" s="7" t="n"/>
+    </row>
+    <row r="405">
+      <c r="M405" s="7" t="n"/>
+      <c r="N405" s="7" t="n"/>
+      <c r="O405" s="7" t="n"/>
+      <c r="P405" s="7" t="n"/>
+    </row>
+    <row r="406">
+      <c r="M406" s="7" t="n"/>
+      <c r="N406" s="7" t="n"/>
+      <c r="O406" s="7" t="n"/>
+      <c r="P406" s="7" t="n"/>
+    </row>
+    <row r="407">
+      <c r="M407" s="7" t="n"/>
+      <c r="N407" s="7" t="n"/>
+      <c r="O407" s="7" t="n"/>
+      <c r="P407" s="7" t="n"/>
+    </row>
+    <row r="408">
+      <c r="M408" s="7" t="n"/>
+      <c r="N408" s="7" t="n"/>
+      <c r="O408" s="7" t="n"/>
+      <c r="P408" s="7" t="n"/>
+    </row>
+    <row r="409">
+      <c r="M409" s="7" t="n"/>
+      <c r="N409" s="7" t="n"/>
+      <c r="O409" s="7" t="n"/>
+      <c r="P409" s="7" t="n"/>
+    </row>
+    <row r="410">
+      <c r="M410" s="7" t="n"/>
+      <c r="N410" s="7" t="n"/>
+      <c r="O410" s="7" t="n"/>
+      <c r="P410" s="7" t="n"/>
+    </row>
+    <row r="411">
+      <c r="M411" s="7" t="n"/>
+      <c r="N411" s="7" t="n"/>
+      <c r="O411" s="7" t="n"/>
+      <c r="P411" s="7" t="n"/>
+    </row>
+    <row r="412">
+      <c r="M412" s="7" t="n"/>
+      <c r="N412" s="7" t="n"/>
+      <c r="O412" s="7" t="n"/>
+      <c r="P412" s="7" t="n"/>
+    </row>
+    <row r="413">
+      <c r="M413" s="7" t="n"/>
+      <c r="N413" s="7" t="n"/>
+      <c r="O413" s="7" t="n"/>
+      <c r="P413" s="7" t="n"/>
+    </row>
+    <row r="414">
+      <c r="M414" s="7" t="n"/>
+      <c r="N414" s="7" t="n"/>
+      <c r="O414" s="7" t="n"/>
+      <c r="P414" s="7" t="n"/>
+    </row>
+    <row r="415">
+      <c r="M415" s="7" t="n"/>
+      <c r="N415" s="7" t="n"/>
+      <c r="O415" s="7" t="n"/>
+      <c r="P415" s="7" t="n"/>
+    </row>
+    <row r="416">
+      <c r="M416" s="7" t="n"/>
+      <c r="N416" s="7" t="n"/>
+      <c r="O416" s="7" t="n"/>
+      <c r="P416" s="7" t="n"/>
+    </row>
+    <row r="417">
+      <c r="M417" s="7" t="n"/>
+      <c r="N417" s="7" t="n"/>
+      <c r="O417" s="7" t="n"/>
+      <c r="P417" s="7" t="n"/>
+    </row>
+    <row r="418">
+      <c r="M418" s="7" t="n"/>
+      <c r="N418" s="7" t="n"/>
+      <c r="O418" s="7" t="n"/>
+      <c r="P418" s="7" t="n"/>
+    </row>
+    <row r="419">
+      <c r="M419" s="7" t="n"/>
+      <c r="N419" s="7" t="n"/>
+      <c r="O419" s="7" t="n"/>
+      <c r="P419" s="7" t="n"/>
+    </row>
+    <row r="420">
+      <c r="M420" s="7" t="n"/>
+      <c r="N420" s="7" t="n"/>
+      <c r="O420" s="7" t="n"/>
+      <c r="P420" s="7" t="n"/>
+    </row>
+    <row r="421">
+      <c r="M421" s="7" t="n"/>
+      <c r="N421" s="7" t="n"/>
+      <c r="O421" s="7" t="n"/>
+      <c r="P421" s="7" t="n"/>
+    </row>
+    <row r="422">
+      <c r="M422" s="7" t="n"/>
+      <c r="N422" s="7" t="n"/>
+      <c r="O422" s="7" t="n"/>
+      <c r="P422" s="7" t="n"/>
+    </row>
+    <row r="423">
+      <c r="M423" s="7" t="n"/>
+      <c r="N423" s="7" t="n"/>
+      <c r="O423" s="7" t="n"/>
+      <c r="P423" s="7" t="n"/>
+    </row>
+    <row r="424">
+      <c r="M424" s="7" t="n"/>
+      <c r="N424" s="7" t="n"/>
+      <c r="O424" s="7" t="n"/>
+      <c r="P424" s="7" t="n"/>
+    </row>
+    <row r="425">
+      <c r="M425" s="7" t="n"/>
+      <c r="N425" s="7" t="n"/>
+      <c r="O425" s="7" t="n"/>
+      <c r="P425" s="7" t="n"/>
+    </row>
+    <row r="426">
+      <c r="M426" s="7" t="n"/>
+      <c r="N426" s="7" t="n"/>
+      <c r="O426" s="7" t="n"/>
+      <c r="P426" s="7" t="n"/>
+    </row>
+    <row r="427">
+      <c r="M427" s="7" t="n"/>
+      <c r="N427" s="7" t="n"/>
+      <c r="O427" s="7" t="n"/>
+      <c r="P427" s="7" t="n"/>
+    </row>
+    <row r="428">
+      <c r="M428" s="7" t="n"/>
+      <c r="N428" s="7" t="n"/>
+      <c r="O428" s="7" t="n"/>
+      <c r="P428" s="7" t="n"/>
+    </row>
+    <row r="429">
+      <c r="M429" s="7" t="n"/>
+      <c r="N429" s="7" t="n"/>
+      <c r="O429" s="7" t="n"/>
+      <c r="P429" s="7" t="n"/>
+    </row>
+    <row r="430">
+      <c r="M430" s="7" t="n"/>
+      <c r="N430" s="7" t="n"/>
+      <c r="O430" s="7" t="n"/>
+      <c r="P430" s="7" t="n"/>
+    </row>
+    <row r="431">
+      <c r="M431" s="7" t="n"/>
+      <c r="N431" s="7" t="n"/>
+      <c r="O431" s="7" t="n"/>
+      <c r="P431" s="7" t="n"/>
+    </row>
+    <row r="432">
+      <c r="M432" s="7" t="n"/>
+      <c r="N432" s="7" t="n"/>
+      <c r="O432" s="7" t="n"/>
+      <c r="P432" s="7" t="n"/>
+    </row>
+    <row r="433">
+      <c r="M433" s="7" t="n"/>
+      <c r="N433" s="7" t="n"/>
+      <c r="O433" s="7" t="n"/>
+      <c r="P433" s="7" t="n"/>
+    </row>
+    <row r="434">
+      <c r="M434" s="7" t="n"/>
+      <c r="N434" s="7" t="n"/>
+      <c r="O434" s="7" t="n"/>
+      <c r="P434" s="7" t="n"/>
+    </row>
+    <row r="435">
+      <c r="M435" s="7" t="n"/>
+      <c r="N435" s="7" t="n"/>
+      <c r="O435" s="7" t="n"/>
+      <c r="P435" s="7" t="n"/>
+    </row>
+    <row r="436">
+      <c r="M436" s="7" t="n"/>
+      <c r="N436" s="7" t="n"/>
+      <c r="O436" s="7" t="n"/>
+      <c r="P436" s="7" t="n"/>
+    </row>
+    <row r="437">
+      <c r="M437" s="7" t="n"/>
+      <c r="N437" s="7" t="n"/>
+      <c r="O437" s="7" t="n"/>
+      <c r="P437" s="7" t="n"/>
+    </row>
+    <row r="438">
+      <c r="M438" s="7" t="n"/>
+      <c r="N438" s="7" t="n"/>
+      <c r="O438" s="7" t="n"/>
+      <c r="P438" s="7" t="n"/>
+    </row>
+    <row r="439">
+      <c r="M439" s="7" t="n"/>
+      <c r="N439" s="7" t="n"/>
+      <c r="O439" s="7" t="n"/>
+      <c r="P439" s="7" t="n"/>
+    </row>
+    <row r="440">
+      <c r="M440" s="7" t="n"/>
+      <c r="N440" s="7" t="n"/>
+      <c r="O440" s="7" t="n"/>
+      <c r="P440" s="7" t="n"/>
+    </row>
+    <row r="441">
+      <c r="M441" s="7" t="n"/>
+      <c r="N441" s="7" t="n"/>
+      <c r="O441" s="7" t="n"/>
+      <c r="P441" s="7" t="n"/>
+    </row>
+    <row r="442">
+      <c r="M442" s="7" t="n"/>
+      <c r="N442" s="7" t="n"/>
+      <c r="O442" s="7" t="n"/>
+      <c r="P442" s="7" t="n"/>
+    </row>
+    <row r="443">
+      <c r="M443" s="7" t="n"/>
+      <c r="N443" s="7" t="n"/>
+      <c r="O443" s="7" t="n"/>
+      <c r="P443" s="7" t="n"/>
+    </row>
+    <row r="444">
+      <c r="M444" s="7" t="n"/>
+      <c r="N444" s="7" t="n"/>
+      <c r="O444" s="7" t="n"/>
+      <c r="P444" s="7" t="n"/>
+    </row>
+    <row r="445">
+      <c r="M445" s="7" t="n"/>
+      <c r="N445" s="7" t="n"/>
+      <c r="O445" s="7" t="n"/>
+      <c r="P445" s="7" t="n"/>
+    </row>
+    <row r="446">
+      <c r="M446" s="7" t="n"/>
+      <c r="N446" s="7" t="n"/>
+      <c r="O446" s="7" t="n"/>
+      <c r="P446" s="7" t="n"/>
+    </row>
+    <row r="447">
+      <c r="M447" s="7" t="n"/>
+      <c r="N447" s="7" t="n"/>
+      <c r="O447" s="7" t="n"/>
+      <c r="P447" s="7" t="n"/>
+    </row>
+    <row r="448">
+      <c r="M448" s="7" t="n"/>
+      <c r="N448" s="7" t="n"/>
+      <c r="O448" s="7" t="n"/>
+      <c r="P448" s="7" t="n"/>
+    </row>
+    <row r="449">
+      <c r="M449" s="7" t="n"/>
+      <c r="N449" s="7" t="n"/>
+      <c r="O449" s="7" t="n"/>
+      <c r="P449" s="7" t="n"/>
+    </row>
+    <row r="450">
+      <c r="M450" s="7" t="n"/>
+      <c r="N450" s="7" t="n"/>
+      <c r="O450" s="7" t="n"/>
+      <c r="P450" s="7" t="n"/>
+    </row>
+    <row r="451">
+      <c r="M451" s="7" t="n"/>
+      <c r="N451" s="7" t="n"/>
+      <c r="O451" s="7" t="n"/>
+      <c r="P451" s="7" t="n"/>
+    </row>
+    <row r="452">
+      <c r="M452" s="7" t="n"/>
+      <c r="N452" s="7" t="n"/>
+      <c r="O452" s="7" t="n"/>
+      <c r="P452" s="7" t="n"/>
+    </row>
+    <row r="453">
+      <c r="M453" s="7" t="n"/>
+      <c r="N453" s="7" t="n"/>
+      <c r="O453" s="7" t="n"/>
+      <c r="P453" s="7" t="n"/>
+    </row>
+    <row r="454">
+      <c r="M454" s="7" t="n"/>
+      <c r="N454" s="7" t="n"/>
+      <c r="O454" s="7" t="n"/>
+      <c r="P454" s="7" t="n"/>
+    </row>
+    <row r="455">
+      <c r="M455" s="7" t="n"/>
+      <c r="N455" s="7" t="n"/>
+      <c r="O455" s="7" t="n"/>
+      <c r="P455" s="7" t="n"/>
+    </row>
+    <row r="456">
+      <c r="M456" s="7" t="n"/>
+      <c r="N456" s="7" t="n"/>
+      <c r="O456" s="7" t="n"/>
+      <c r="P456" s="7" t="n"/>
+    </row>
+    <row r="457">
+      <c r="M457" s="7" t="n"/>
+      <c r="N457" s="7" t="n"/>
+      <c r="O457" s="7" t="n"/>
+      <c r="P457" s="7" t="n"/>
+    </row>
+    <row r="458">
+      <c r="M458" s="7" t="n"/>
+      <c r="N458" s="7" t="n"/>
+      <c r="O458" s="7" t="n"/>
+      <c r="P458" s="7" t="n"/>
+    </row>
+    <row r="459">
+      <c r="M459" s="7" t="n"/>
+      <c r="N459" s="7" t="n"/>
+      <c r="O459" s="7" t="n"/>
+      <c r="P459" s="7" t="n"/>
+    </row>
+    <row r="460">
+      <c r="M460" s="7" t="n"/>
+      <c r="N460" s="7" t="n"/>
+      <c r="O460" s="7" t="n"/>
+      <c r="P460" s="7" t="n"/>
+    </row>
+    <row r="461">
+      <c r="M461" s="7" t="n"/>
+      <c r="N461" s="7" t="n"/>
+      <c r="O461" s="7" t="n"/>
+      <c r="P461" s="7" t="n"/>
+    </row>
+    <row r="462">
+      <c r="M462" s="7" t="n"/>
+      <c r="N462" s="7" t="n"/>
+      <c r="O462" s="7" t="n"/>
+      <c r="P462" s="7" t="n"/>
+    </row>
+    <row r="463">
+      <c r="M463" s="7" t="n"/>
+      <c r="N463" s="7" t="n"/>
+      <c r="O463" s="7" t="n"/>
+      <c r="P463" s="7" t="n"/>
+    </row>
+    <row r="464">
+      <c r="M464" s="7" t="n"/>
+      <c r="N464" s="7" t="n"/>
+      <c r="O464" s="7" t="n"/>
+      <c r="P464" s="7" t="n"/>
+    </row>
+    <row r="465">
+      <c r="M465" s="7" t="n"/>
+      <c r="N465" s="7" t="n"/>
+      <c r="O465" s="7" t="n"/>
+      <c r="P465" s="7" t="n"/>
+    </row>
+    <row r="466">
+      <c r="M466" s="7" t="n"/>
+      <c r="N466" s="7" t="n"/>
+      <c r="O466" s="7" t="n"/>
+      <c r="P466" s="7" t="n"/>
+    </row>
+    <row r="467">
+      <c r="M467" s="7" t="n"/>
+      <c r="N467" s="7" t="n"/>
+      <c r="O467" s="7" t="n"/>
+      <c r="P467" s="7" t="n"/>
+    </row>
+    <row r="468">
+      <c r="M468" s="7" t="n"/>
+      <c r="N468" s="7" t="n"/>
+      <c r="O468" s="7" t="n"/>
+      <c r="P468" s="7" t="n"/>
+    </row>
+    <row r="469">
+      <c r="M469" s="7" t="n"/>
+      <c r="N469" s="7" t="n"/>
+      <c r="O469" s="7" t="n"/>
+      <c r="P469" s="7" t="n"/>
+    </row>
+    <row r="470">
+      <c r="M470" s="7" t="n"/>
+      <c r="N470" s="7" t="n"/>
+      <c r="O470" s="7" t="n"/>
+      <c r="P470" s="7" t="n"/>
+    </row>
+    <row r="471">
+      <c r="M471" s="7" t="n"/>
+      <c r="N471" s="7" t="n"/>
+      <c r="O471" s="7" t="n"/>
+      <c r="P471" s="7" t="n"/>
+    </row>
+    <row r="472">
+      <c r="M472" s="7" t="n"/>
+      <c r="N472" s="7" t="n"/>
+      <c r="O472" s="7" t="n"/>
+      <c r="P472" s="7" t="n"/>
+    </row>
+    <row r="473">
+      <c r="M473" s="7" t="n"/>
+      <c r="N473" s="7" t="n"/>
+      <c r="O473" s="7" t="n"/>
+      <c r="P473" s="7" t="n"/>
+    </row>
+    <row r="474">
+      <c r="M474" s="7" t="n"/>
+      <c r="N474" s="7" t="n"/>
+      <c r="O474" s="7" t="n"/>
+      <c r="P474" s="7" t="n"/>
+    </row>
+    <row r="475">
+      <c r="M475" s="7" t="n"/>
+      <c r="N475" s="7" t="n"/>
+      <c r="O475" s="7" t="n"/>
+      <c r="P475" s="7" t="n"/>
+    </row>
+    <row r="476">
+      <c r="M476" s="7" t="n"/>
+      <c r="N476" s="7" t="n"/>
+      <c r="O476" s="7" t="n"/>
+      <c r="P476" s="7" t="n"/>
+    </row>
+    <row r="477">
+      <c r="M477" s="7" t="n"/>
+      <c r="N477" s="7" t="n"/>
+      <c r="O477" s="7" t="n"/>
+      <c r="P477" s="7" t="n"/>
+    </row>
+    <row r="478">
+      <c r="M478" s="7" t="n"/>
+      <c r="N478" s="7" t="n"/>
+      <c r="O478" s="7" t="n"/>
+      <c r="P478" s="7" t="n"/>
+    </row>
+    <row r="479">
+      <c r="M479" s="7" t="n"/>
+      <c r="N479" s="7" t="n"/>
+      <c r="O479" s="7" t="n"/>
+      <c r="P479" s="7" t="n"/>
+    </row>
+    <row r="480">
+      <c r="M480" s="7" t="n"/>
+      <c r="N480" s="7" t="n"/>
+      <c r="O480" s="7" t="n"/>
+      <c r="P480" s="7" t="n"/>
+    </row>
+    <row r="481">
+      <c r="M481" s="7" t="n"/>
+      <c r="N481" s="7" t="n"/>
+      <c r="O481" s="7" t="n"/>
+      <c r="P481" s="7" t="n"/>
+    </row>
+    <row r="482">
+      <c r="M482" s="7" t="n"/>
+      <c r="N482" s="7" t="n"/>
+      <c r="O482" s="7" t="n"/>
+      <c r="P482" s="7" t="n"/>
+    </row>
+    <row r="483">
+      <c r="M483" s="7" t="n"/>
+      <c r="N483" s="7" t="n"/>
+      <c r="O483" s="7" t="n"/>
+      <c r="P483" s="7" t="n"/>
+    </row>
+    <row r="484">
+      <c r="M484" s="7" t="n"/>
+      <c r="N484" s="7" t="n"/>
+      <c r="O484" s="7" t="n"/>
+      <c r="P484" s="7" t="n"/>
+    </row>
+    <row r="485">
+      <c r="M485" s="7" t="n"/>
+      <c r="N485" s="7" t="n"/>
+      <c r="O485" s="7" t="n"/>
+      <c r="P485" s="7" t="n"/>
+    </row>
+    <row r="486">
+      <c r="M486" s="7" t="n"/>
+      <c r="N486" s="7" t="n"/>
+      <c r="O486" s="7" t="n"/>
+      <c r="P486" s="7" t="n"/>
+    </row>
+    <row r="487">
+      <c r="M487" s="7" t="n"/>
+      <c r="N487" s="7" t="n"/>
+      <c r="O487" s="7" t="n"/>
+      <c r="P487" s="7" t="n"/>
+    </row>
+    <row r="488">
+      <c r="M488" s="7" t="n"/>
+      <c r="N488" s="7" t="n"/>
+      <c r="O488" s="7" t="n"/>
+      <c r="P488" s="7" t="n"/>
+    </row>
+    <row r="489">
+      <c r="M489" s="7" t="n"/>
+      <c r="N489" s="7" t="n"/>
+      <c r="O489" s="7" t="n"/>
+      <c r="P489" s="7" t="n"/>
+    </row>
+    <row r="490">
+      <c r="M490" s="7" t="n"/>
+      <c r="N490" s="7" t="n"/>
+      <c r="O490" s="7" t="n"/>
+      <c r="P490" s="7" t="n"/>
+    </row>
+    <row r="491">
+      <c r="M491" s="7" t="n"/>
+      <c r="N491" s="7" t="n"/>
+      <c r="O491" s="7" t="n"/>
+      <c r="P491" s="7" t="n"/>
+    </row>
+    <row r="492">
+      <c r="M492" s="7" t="n"/>
+      <c r="N492" s="7" t="n"/>
+      <c r="O492" s="7" t="n"/>
+      <c r="P492" s="7" t="n"/>
+    </row>
+    <row r="493">
+      <c r="M493" s="7" t="n"/>
+      <c r="N493" s="7" t="n"/>
+      <c r="O493" s="7" t="n"/>
+      <c r="P493" s="7" t="n"/>
+    </row>
+    <row r="494">
+      <c r="M494" s="7" t="n"/>
+      <c r="N494" s="7" t="n"/>
+      <c r="O494" s="7" t="n"/>
+      <c r="P494" s="7" t="n"/>
+    </row>
+    <row r="495">
+      <c r="M495" s="7" t="n"/>
+      <c r="N495" s="7" t="n"/>
+      <c r="O495" s="7" t="n"/>
+      <c r="P495" s="7" t="n"/>
+    </row>
+    <row r="496">
+      <c r="M496" s="7" t="n"/>
+      <c r="N496" s="7" t="n"/>
+      <c r="O496" s="7" t="n"/>
+      <c r="P496" s="7" t="n"/>
+    </row>
+    <row r="497">
+      <c r="M497" s="7" t="n"/>
+      <c r="N497" s="7" t="n"/>
+      <c r="O497" s="7" t="n"/>
+      <c r="P497" s="7" t="n"/>
+    </row>
+    <row r="498">
+      <c r="M498" s="7" t="n"/>
+      <c r="N498" s="7" t="n"/>
+      <c r="O498" s="7" t="n"/>
+      <c r="P498" s="7" t="n"/>
+    </row>
+    <row r="499">
+      <c r="M499" s="7" t="n"/>
+      <c r="N499" s="7" t="n"/>
+      <c r="O499" s="7" t="n"/>
+      <c r="P499" s="7" t="n"/>
+    </row>
+    <row r="500">
+      <c r="M500" s="7" t="n"/>
+      <c r="N500" s="7" t="n"/>
+      <c r="O500" s="7" t="n"/>
+      <c r="P500" s="7" t="n"/>
+    </row>
+    <row r="501">
+      <c r="M501" s="7" t="n"/>
+      <c r="N501" s="7" t="n"/>
+      <c r="O501" s="7" t="n"/>
+      <c r="P501" s="7" t="n"/>
+    </row>
+    <row r="502">
+      <c r="M502" s="7" t="n"/>
+      <c r="N502" s="7" t="n"/>
+      <c r="O502" s="7" t="n"/>
+      <c r="P502" s="7" t="n"/>
+    </row>
+    <row r="503">
+      <c r="M503" s="7" t="n"/>
+      <c r="N503" s="7" t="n"/>
+      <c r="O503" s="7" t="n"/>
+      <c r="P503" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -934,42 +4155,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Change Type</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>Risk Level</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>CAB Approval</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>Validation Status</t>
         </is>
       </c>
-      <c r="M1" s="7" t="inlineStr">
+      <c r="M1" s="8" t="inlineStr">
         <is>
           <t>Change Category</t>
         </is>
       </c>
-      <c r="O1" s="7" t="inlineStr">
+      <c r="O1" s="8" t="inlineStr">
         <is>
           <t>Rollback Plan</t>
         </is>

</xml_diff>

<commit_message>
fix(generator): align sample changes with registered CI and asset IDs
</commit_message>
<xml_diff>
--- a/docs/engineering/change-management/PO-CHANGE-REGISTER_v1.0.xlsx
+++ b/docs/engineering/change-management/PO-CHANGE-REGISTER_v1.0.xlsx
@@ -842,12 +842,12 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>CI-NET-001</t>
+          <t>CI-003</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>AST-NET-001</t>
+          <t>AST-003</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
@@ -927,12 +927,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CI-SRV-001</t>
+          <t>CI-004</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>AST-SRV-001</t>
+          <t>AST-004</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -982,12 +982,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rotate Cloud Service Credentials</t>
+          <t>Update Home Assistant Service Credentials</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Cloud</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1012,12 +1012,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>CI-CLD-001</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>AST-CLD-001</t>
+          <t>CI-006</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">

</xml_diff>